<commit_message>
Update flooring costs: new box counts, stair parts, 5% contractor discount
- Box quantities from re-priced Floor & Decor cart: Sapelo Shore 66,
  Big Sur 60, Gunstock Oak 64
- Add stair nose trim (7 x $29.99) and stair risers (13 x $20) material lines
- Add 5% contractor discount line on all materials; sales tax now estimated
  on the discounted amount
- Refactor project-tab layout to computed row positions so the basis link
  and HLOOKUP offsets track structural changes automatically

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KP5NvhWhWoi9eWvxEnz5vK
</commit_message>
<xml_diff>
--- a/4-Indian-Brook-House-Tracker.xlsx
+++ b/4-Indian-Brook-House-Tracker.xlsx
@@ -671,7 +671,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2nd Floor Flooring</t>
@@ -679,7 +679,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>First project. Compare the 3 Floor &amp; Decor plank options, pick one in 'Selected option' (yellow cell), and the budget fills in automatically. Log payments in the cost log at the bottom — actuals and the Basis Tracker update themselves.</t>
+          <t>First project. Compare the 3 Floor &amp; Decor plank options (incl. underlayment, stair nose &amp; risers, 5% contractor discount, est. tax, and Footprints labor), pick one in 'Selected option' (yellow cell), and the budget fills in automatically. Log payments in the cost log at the bottom — actuals and the Basis Tracker update themselves.</t>
         </is>
       </c>
     </row>
@@ -691,11 +691,11 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>For the next project: right-click the tab &gt; Duplicate, rename it, fill in your options/quotes, then add a row in the Basis Tracker improvements table pointing at the new tab's cell C37 (its Actual total).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
+          <t>For the next project: right-click the tab &gt; Duplicate, rename it, fill in your options/quotes, then add a row in the Basis Tracker improvements table pointing at the new tab's cell C43 (its Actual total).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Sources</t>
@@ -703,7 +703,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Labor: Footprints Floors of Central MA proposal #25584 (6/30/2026) — $9,057.60, materials excluded. Materials: Floor &amp; Decor Waltham cart — Sapelo Shore / Big Sur / Gunstock Oak + Sentinel underlayment.</t>
+          <t>Labor: Footprints Floors of Central MA proposal #25584 (6/30/2026) — $9,057.60, materials excluded. Materials: Floor &amp; Decor Waltham cart (7/2026) — Sapelo Shore / Big Sur / Gunstock Oak + Sentinel underlayment, plus 7 stair noses @ $29.99 and 13 risers @ $20; 5% contractor discount on materials.</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="E21" s="14">
-        <f>'2nd Floor Flooring'!C37</f>
+        <f>'2nd Floor Flooring'!C43</f>
         <v/>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Floor &amp; Decor, Waltham MA (cart priced 7/2026)</t>
+          <t>Floor &amp; Decor, Waltham MA (cart re-priced 7/2026); 5% materials discount through flooring contractor</t>
         </is>
       </c>
     </row>
@@ -1375,13 +1375,13 @@
         </is>
       </c>
       <c r="B16" s="29" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C16" s="29" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E16" s="12" t="n"/>
     </row>
@@ -1434,24 +1434,24 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Est. sales tax (6.25% MA, materials)</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B19" s="28">
-        <f>(B17+B18)*0.0625</f>
+        <f>7*29.99</f>
         <v/>
       </c>
       <c r="C19" s="28">
-        <f>(C17+C18)*0.0625</f>
+        <f>7*29.99</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>(D17+D18)*0.0625</f>
+        <f>7*29.99</f>
         <v/>
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>Estimate on materials only; replace with the actual receipt tax when purchased.</t>
+          <t>7 stair noses x $29.99.</t>
         </is>
       </c>
       <c r="F19" s="10" t="n"/>
@@ -1460,21 +1460,24 @@
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
-        </is>
-      </c>
-      <c r="B20" s="28" t="n">
-        <v>2642.3</v>
-      </c>
-      <c r="C20" s="28" t="n">
-        <v>2642.3</v>
-      </c>
-      <c r="D20" s="28" t="n">
-        <v>2642.3</v>
+          <t>Stair risers</t>
+        </is>
+      </c>
+      <c r="B20" s="28">
+        <f>13*20</f>
+        <v/>
+      </c>
+      <c r="C20" s="28">
+        <f>13*20</f>
+        <v/>
+      </c>
+      <c r="D20" s="28">
+        <f>13*20</f>
+        <v/>
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>Footprints: demo carpet, remove &amp; return baseboards, trash removal.</t>
+          <t>13 risers x $20.00.</t>
         </is>
       </c>
       <c r="F20" s="10" t="n"/>
@@ -1483,21 +1486,24 @@
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>Labor — install</t>
-        </is>
-      </c>
-      <c r="B21" s="28" t="n">
-        <v>4535.3</v>
-      </c>
-      <c r="C21" s="28" t="n">
-        <v>4535.3</v>
-      </c>
-      <c r="D21" s="28" t="n">
-        <v>4535.3</v>
+          <t>Contractor discount on materials (5%)</t>
+        </is>
+      </c>
+      <c r="B21" s="28">
+        <f>-0.05*SUM(B17:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="28">
+        <f>-0.05*SUM(C17:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="28">
+        <f>-0.05*SUM(D17:D20)</f>
+        <v/>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Footprints: install click-lock floating floor.</t>
+          <t>5% off all materials through the flooring contractor.</t>
         </is>
       </c>
       <c r="F21" s="10" t="n"/>
@@ -1506,170 +1512,173 @@
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>Labor — stairs (treads &amp; risers)</t>
-        </is>
-      </c>
-      <c r="B22" s="28" t="n">
-        <v>1880</v>
-      </c>
-      <c r="C22" s="28" t="n">
-        <v>1880</v>
-      </c>
-      <c r="D22" s="28" t="n">
-        <v>1880</v>
-      </c>
-      <c r="E22" s="27" t="inlineStr">
-        <is>
-          <t>Footprints: treads (open 1 side) + risers.</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="11" t="n"/>
+          <t>Est. sales tax (6.25% MA, materials)</t>
+        </is>
+      </c>
+      <c r="B22" s="28">
+        <f>SUM(B17:B21)*0.0625</f>
+        <v/>
+      </c>
+      <c r="C22" s="28">
+        <f>SUM(C17:C21)*0.0625</f>
+        <v/>
+      </c>
+      <c r="D22" s="28">
+        <f>SUM(D17:D21)*0.0625</f>
+        <v/>
+      </c>
+      <c r="E22" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
-        <is>
-          <t>TOTAL ESTIMATED</t>
-        </is>
-      </c>
-      <c r="B23" s="31">
-        <f>SUM(B17:B22)</f>
-        <v/>
-      </c>
-      <c r="C23" s="31">
-        <f>SUM(C17:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="31">
-        <f>SUM(D17:D22)</f>
-        <v/>
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>Labor — demo &amp; disposal</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="n">
+        <v>2642.3</v>
+      </c>
+      <c r="C23" s="28" t="n">
+        <v>2642.3</v>
+      </c>
+      <c r="D23" s="28" t="n">
+        <v>2642.3</v>
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>Labor $9,057.60 is identical across options, so the spread comes entirely from the plank you pick.</t>
+          <t>Footprints: demo carpet, remove &amp; return baseboards, trash removal.</t>
         </is>
       </c>
       <c r="F23" s="10" t="n"/>
       <c r="G23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>Labor — install</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="n">
+        <v>4535.3</v>
+      </c>
+      <c r="C24" s="28" t="n">
+        <v>4535.3</v>
+      </c>
+      <c r="D24" s="28" t="n">
+        <v>4535.3</v>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>Footprints: install click-lock floating floor.</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="11" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>Labor — stairs (treads &amp; risers)</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="n">
+        <v>1880</v>
+      </c>
+      <c r="C25" s="28" t="n">
+        <v>1880</v>
+      </c>
+      <c r="D25" s="28" t="n">
+        <v>1880</v>
+      </c>
+      <c r="E25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>TOTAL ESTIMATED</t>
+        </is>
+      </c>
+      <c r="B26" s="31">
+        <f>SUM(B17:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="31">
+        <f>SUM(C17:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31">
+        <f>SUM(D17:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>Labor $9,057.60 is identical across options, so the spread comes entirely from the plank you pick.</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t>Premium vs. cheapest option</t>
         </is>
       </c>
-      <c r="B24" s="33">
-        <f>B23-MIN($B$23:$D$23)</f>
-        <v/>
-      </c>
-      <c r="C24" s="33">
-        <f>C23-MIN($B$23:$D$23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="33">
-        <f>D23-MIN($B$23:$D$23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="12" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="B27" s="33">
+        <f>B26-MIN($B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="33">
+        <f>C26-MIN($B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="33">
+        <f>D26-MIN($B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="12" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>STEP 2 — BUDGET vs. ACTUAL  (budget auto-fills from the selected option)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Actual (from cost log)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Flooring materials</t>
-        </is>
-      </c>
-      <c r="B28" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,5,FALSE))</f>
-        <v/>
-      </c>
-      <c r="C28" s="14">
-        <f>SUMIF($D$42:$D$140,$A28,$E$42:$E$140)</f>
-        <v/>
-      </c>
-      <c r="D28" s="14">
-        <f>IF(B28="","",B28-C28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Underlayment &amp; supplies</t>
-        </is>
-      </c>
-      <c r="B29" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,6,FALSE))</f>
-        <v/>
-      </c>
-      <c r="C29" s="14">
-        <f>SUMIF($D$42:$D$140,$A29,$E$42:$E$140)</f>
-        <v/>
-      </c>
-      <c r="D29" s="14">
-        <f>IF(B29="","",B29-C29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Sales tax</t>
-        </is>
-      </c>
-      <c r="B30" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,7,FALSE))</f>
-        <v/>
-      </c>
-      <c r="C30" s="14">
-        <f>SUMIF($D$42:$D$140,$A30,$E$42:$E$140)</f>
-        <v/>
-      </c>
-      <c r="D30" s="14">
-        <f>IF(B30="","",B30-C30)</f>
-        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Flooring materials</t>
         </is>
       </c>
       <c r="B31" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,8,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,5,FALSE))</f>
         <v/>
       </c>
       <c r="C31" s="14">
-        <f>SUMIF($D$42:$D$140,$A31,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A31,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D31" s="14">
@@ -1680,15 +1689,15 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Labor — install</t>
+          <t>Underlayment &amp; supplies</t>
         </is>
       </c>
       <c r="B32" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,9,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,6,FALSE))</f>
         <v/>
       </c>
       <c r="C32" s="14">
-        <f>SUMIF($D$42:$D$140,$A32,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A32,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D32" s="14">
@@ -1699,15 +1708,15 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Labor — stairs</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B33" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,10,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,7,FALSE))</f>
         <v/>
       </c>
       <c r="C33" s="14">
-        <f>SUMIF($D$42:$D$140,$A33,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A33,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D33" s="14">
@@ -1718,12 +1727,15 @@
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Permits &amp; fees</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="n"/>
+          <t>Stair risers</t>
+        </is>
+      </c>
+      <c r="B34" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,8,FALSE))</f>
+        <v/>
+      </c>
       <c r="C34" s="14">
-        <f>SUMIF($D$42:$D$140,$A34,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A34,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D34" s="14">
@@ -1734,12 +1746,15 @@
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="n"/>
+          <t>Contractor discount</t>
+        </is>
+      </c>
+      <c r="B35" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,9,FALSE))</f>
+        <v/>
+      </c>
       <c r="C35" s="14">
-        <f>SUMIF($D$42:$D$140,$A35,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A35,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D35" s="14">
@@ -1750,142 +1765,196 @@
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
+          <t>Sales tax</t>
+        </is>
+      </c>
+      <c r="B36" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,10,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C36" s="14">
+        <f>SUMIF($D$48:$D$147,$A36,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D36" s="14">
+        <f>IF(B36="","",B36-C36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Labor — demo &amp; disposal</t>
+        </is>
+      </c>
+      <c r="B37" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,11,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C37" s="14">
+        <f>SUMIF($D$48:$D$147,$A37,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D37" s="14">
+        <f>IF(B37="","",B37-C37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Labor — install</t>
+        </is>
+      </c>
+      <c r="B38" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,12,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C38" s="14">
+        <f>SUMIF($D$48:$D$147,$A38,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D38" s="14">
+        <f>IF(B38="","",B38-C38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Labor — stairs</t>
+        </is>
+      </c>
+      <c r="B39" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,13,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C39" s="14">
+        <f>SUMIF($D$48:$D$147,$A39,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D39" s="14">
+        <f>IF(B39="","",B39-C39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Permits &amp; fees</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="n"/>
+      <c r="C40" s="14">
+        <f>SUMIF($D$48:$D$147,$A40,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D40" s="14">
+        <f>IF(B40="","",B40-C40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14">
+        <f>SUMIF($D$48:$D$147,$A41,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D41" s="14">
+        <f>IF(B41="","",B41-C41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
           <t>Contingency</t>
         </is>
       </c>
-      <c r="B36" s="14">
-        <f>SUM(B28:B35)*$B$9</f>
-        <v/>
-      </c>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14">
-        <f>B36-C36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
+      <c r="B42" s="14">
+        <f>SUM(B31:B41)*$B$9</f>
+        <v/>
+      </c>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B37" s="34">
-        <f>SUM(B28:B36)</f>
-        <v/>
-      </c>
-      <c r="C37" s="34">
-        <f>SUM(C28:C36)</f>
-        <v/>
-      </c>
-      <c r="D37" s="34">
-        <f>B37-C37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>The Actual total (C37) is what feeds the Basis Tracker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="B43" s="34">
+        <f>SUM(B31:B42)</f>
+        <v/>
+      </c>
+      <c r="C43" s="34">
+        <f>SUM(C31:C42)</f>
+        <v/>
+      </c>
+      <c r="D43" s="34">
+        <f>B43-C43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>The Actual total (C43) is what feeds the Basis Tracker. Log receipts net of discount, or log the discount as a negative amount under 'Contractor discount'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>STEP 3 — COST LOG  (record every payment; Actuals above update automatically)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C47" s="9" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D47" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Payment method</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G47" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="n"/>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="12" t="n"/>
-      <c r="G42" s="12" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="12" t="n"/>
-      <c r="G43" s="12" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n"/>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="12" t="n"/>
-      <c r="G44" s="12" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n"/>
-      <c r="B45" s="12" t="n"/>
-      <c r="C45" s="12" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="12" t="n"/>
-      <c r="G45" s="12" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n"/>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="14" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="n"/>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
@@ -2724,25 +2793,89 @@
       <c r="F140" s="12" t="n"/>
       <c r="G140" s="12" t="n"/>
     </row>
+    <row r="141">
+      <c r="A141" s="8" t="n"/>
+      <c r="B141" s="12" t="n"/>
+      <c r="C141" s="12" t="n"/>
+      <c r="D141" s="12" t="n"/>
+      <c r="E141" s="14" t="n"/>
+      <c r="F141" s="12" t="n"/>
+      <c r="G141" s="12" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="n"/>
+      <c r="B142" s="12" t="n"/>
+      <c r="C142" s="12" t="n"/>
+      <c r="D142" s="12" t="n"/>
+      <c r="E142" s="14" t="n"/>
+      <c r="F142" s="12" t="n"/>
+      <c r="G142" s="12" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="8" t="n"/>
+      <c r="B143" s="12" t="n"/>
+      <c r="C143" s="12" t="n"/>
+      <c r="D143" s="12" t="n"/>
+      <c r="E143" s="14" t="n"/>
+      <c r="F143" s="12" t="n"/>
+      <c r="G143" s="12" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="n"/>
+      <c r="B144" s="12" t="n"/>
+      <c r="C144" s="12" t="n"/>
+      <c r="D144" s="12" t="n"/>
+      <c r="E144" s="14" t="n"/>
+      <c r="F144" s="12" t="n"/>
+      <c r="G144" s="12" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="8" t="n"/>
+      <c r="B145" s="12" t="n"/>
+      <c r="C145" s="12" t="n"/>
+      <c r="D145" s="12" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="12" t="n"/>
+      <c r="G145" s="12" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="n"/>
+      <c r="B146" s="12" t="n"/>
+      <c r="C146" s="12" t="n"/>
+      <c r="D146" s="12" t="n"/>
+      <c r="E146" s="14" t="n"/>
+      <c r="F146" s="12" t="n"/>
+      <c r="G146" s="12" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="8" t="n"/>
+      <c r="B147" s="12" t="n"/>
+      <c r="C147" s="12" t="n"/>
+      <c r="D147" s="12" t="n"/>
+      <c r="E147" s="14" t="n"/>
+      <c r="F147" s="12" t="n"/>
+      <c r="G147" s="12" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="E26:G26"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="E22:G22"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="E18:G18"/>
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="B9:F9"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="E24:G24"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E20:G20"/>
   </mergeCells>
@@ -2753,8 +2886,8 @@
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=$B$13:$D$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=$A$28:$A$35</formula1>
+    <dataValidation sqref="D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=$A$31:$A$41</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2768,7 +2901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2790,7 +2923,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>How to use: right-click the tab &gt; Duplicate. Rename it, fill in options &amp; quotes, then add one row for it in the Basis Tracker improvements table pointing at the new tab's Actual total (cell C37).</t>
+          <t>How to use: right-click the tab &gt; Duplicate. Rename it, fill in options &amp; quotes, then add one row for it in the Basis Tracker improvements table pointing at the new tab's Actual total (cell C43).</t>
         </is>
       </c>
     </row>
@@ -2956,27 +3089,24 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Est. sales tax (6.25% MA, materials)</t>
-        </is>
-      </c>
-      <c r="B19" s="28">
-        <f>(B17+B18)*0.0625</f>
-        <v/>
-      </c>
-      <c r="C19" s="28">
-        <f>(C17+C18)*0.0625</f>
-        <v/>
-      </c>
-      <c r="D19" s="28">
-        <f>(D17+D18)*0.0625</f>
-        <v/>
-      </c>
-      <c r="E19" s="12" t="n"/>
+          <t>Stair nose trim</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr"/>
+      <c r="C19" s="28" t="inlineStr"/>
+      <c r="D19" s="28" t="inlineStr"/>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>Rename these two rows for whatever extra materials the project needs.</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Stair risers</t>
         </is>
       </c>
       <c r="B20" s="28" t="inlineStr"/>
@@ -2987,169 +3117,163 @@
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>Labor — install</t>
-        </is>
-      </c>
-      <c r="B21" s="28" t="inlineStr"/>
-      <c r="C21" s="28" t="inlineStr"/>
-      <c r="D21" s="28" t="inlineStr"/>
+          <t>Contractor discount on materials (0%)</t>
+        </is>
+      </c>
+      <c r="B21" s="28">
+        <f>-0.0*SUM(B17:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="28">
+        <f>-0.0*SUM(C17:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="28">
+        <f>-0.0*SUM(D17:D20)</f>
+        <v/>
+      </c>
       <c r="E21" s="12" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
+          <t>Est. sales tax (6.25% MA, materials)</t>
+        </is>
+      </c>
+      <c r="B22" s="28">
+        <f>SUM(B17:B21)*0.0625</f>
+        <v/>
+      </c>
+      <c r="C22" s="28">
+        <f>SUM(C17:C21)*0.0625</f>
+        <v/>
+      </c>
+      <c r="D22" s="28">
+        <f>SUM(D17:D21)*0.0625</f>
+        <v/>
+      </c>
+      <c r="E22" s="12" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>Labor — demo &amp; disposal</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="inlineStr"/>
+      <c r="C23" s="28" t="inlineStr"/>
+      <c r="D23" s="28" t="inlineStr"/>
+      <c r="E23" s="12" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>Labor — install</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="inlineStr"/>
+      <c r="C24" s="28" t="inlineStr"/>
+      <c r="D24" s="28" t="inlineStr"/>
+      <c r="E24" s="12" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
           <t>Labor — stairs (treads &amp; risers)</t>
         </is>
       </c>
-      <c r="B22" s="28" t="inlineStr"/>
-      <c r="C22" s="28" t="inlineStr"/>
-      <c r="D22" s="28" t="inlineStr"/>
-      <c r="E22" s="12" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="B25" s="28" t="inlineStr"/>
+      <c r="C25" s="28" t="inlineStr"/>
+      <c r="D25" s="28" t="inlineStr"/>
+      <c r="E25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED</t>
         </is>
       </c>
-      <c r="B23" s="31">
-        <f>SUM(B17:B22)</f>
-        <v/>
-      </c>
-      <c r="C23" s="31">
-        <f>SUM(C17:C22)</f>
-        <v/>
-      </c>
-      <c r="D23" s="31">
-        <f>SUM(D17:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="27" t="inlineStr">
+      <c r="B26" s="31">
+        <f>SUM(B17:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="31">
+        <f>SUM(C17:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="31">
+        <f>SUM(D17:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>Compare options here, pick one in 'Selected option' above, and the budget below fills itself in.</t>
         </is>
       </c>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="11" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t>Premium vs. cheapest option</t>
         </is>
       </c>
-      <c r="B24" s="33">
-        <f>B23-MIN($B$23:$D$23)</f>
-        <v/>
-      </c>
-      <c r="C24" s="33">
-        <f>C23-MIN($B$23:$D$23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="33">
-        <f>D23-MIN($B$23:$D$23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="12" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="B27" s="33">
+        <f>B26-MIN($B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="33">
+        <f>C26-MIN($B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="33">
+        <f>D26-MIN($B$26:$D$26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="12" t="n"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>STEP 2 — BUDGET vs. ACTUAL  (budget auto-fills from the selected option)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Actual (from cost log)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Remaining</t>
         </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Flooring materials</t>
-        </is>
-      </c>
-      <c r="B28" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,5,FALSE))</f>
-        <v/>
-      </c>
-      <c r="C28" s="14">
-        <f>SUMIF($D$42:$D$140,$A28,$E$42:$E$140)</f>
-        <v/>
-      </c>
-      <c r="D28" s="14">
-        <f>IF(B28="","",B28-C28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Underlayment &amp; supplies</t>
-        </is>
-      </c>
-      <c r="B29" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,6,FALSE))</f>
-        <v/>
-      </c>
-      <c r="C29" s="14">
-        <f>SUMIF($D$42:$D$140,$A29,$E$42:$E$140)</f>
-        <v/>
-      </c>
-      <c r="D29" s="14">
-        <f>IF(B29="","",B29-C29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Sales tax</t>
-        </is>
-      </c>
-      <c r="B30" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,7,FALSE))</f>
-        <v/>
-      </c>
-      <c r="C30" s="14">
-        <f>SUMIF($D$42:$D$140,$A30,$E$42:$E$140)</f>
-        <v/>
-      </c>
-      <c r="D30" s="14">
-        <f>IF(B30="","",B30-C30)</f>
-        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Flooring materials</t>
         </is>
       </c>
       <c r="B31" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,8,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,5,FALSE))</f>
         <v/>
       </c>
       <c r="C31" s="14">
-        <f>SUMIF($D$42:$D$140,$A31,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A31,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D31" s="14">
@@ -3160,15 +3284,15 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Labor — install</t>
+          <t>Underlayment &amp; supplies</t>
         </is>
       </c>
       <c r="B32" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,9,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,6,FALSE))</f>
         <v/>
       </c>
       <c r="C32" s="14">
-        <f>SUMIF($D$42:$D$140,$A32,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A32,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D32" s="14">
@@ -3179,15 +3303,15 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Labor — stairs</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B33" s="14">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$23,10,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,7,FALSE))</f>
         <v/>
       </c>
       <c r="C33" s="14">
-        <f>SUMIF($D$42:$D$140,$A33,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A33,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D33" s="14">
@@ -3198,12 +3322,15 @@
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Permits &amp; fees</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="n"/>
+          <t>Stair risers</t>
+        </is>
+      </c>
+      <c r="B34" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,8,FALSE))</f>
+        <v/>
+      </c>
       <c r="C34" s="14">
-        <f>SUMIF($D$42:$D$140,$A34,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A34,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D34" s="14">
@@ -3214,12 +3341,15 @@
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="n"/>
+          <t>Contractor discount</t>
+        </is>
+      </c>
+      <c r="B35" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,9,FALSE))</f>
+        <v/>
+      </c>
       <c r="C35" s="14">
-        <f>SUMIF($D$42:$D$140,$A35,$E$42:$E$140)</f>
+        <f>SUMIF($D$48:$D$147,$A35,$E$48:$E$147)</f>
         <v/>
       </c>
       <c r="D35" s="14">
@@ -3230,142 +3360,196 @@
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
+          <t>Sales tax</t>
+        </is>
+      </c>
+      <c r="B36" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,10,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C36" s="14">
+        <f>SUMIF($D$48:$D$147,$A36,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D36" s="14">
+        <f>IF(B36="","",B36-C36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Labor — demo &amp; disposal</t>
+        </is>
+      </c>
+      <c r="B37" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,11,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C37" s="14">
+        <f>SUMIF($D$48:$D$147,$A37,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D37" s="14">
+        <f>IF(B37="","",B37-C37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Labor — install</t>
+        </is>
+      </c>
+      <c r="B38" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,12,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C38" s="14">
+        <f>SUMIF($D$48:$D$147,$A38,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D38" s="14">
+        <f>IF(B38="","",B38-C38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Labor — stairs</t>
+        </is>
+      </c>
+      <c r="B39" s="14">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,13,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C39" s="14">
+        <f>SUMIF($D$48:$D$147,$A39,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D39" s="14">
+        <f>IF(B39="","",B39-C39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Permits &amp; fees</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="n"/>
+      <c r="C40" s="14">
+        <f>SUMIF($D$48:$D$147,$A40,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D40" s="14">
+        <f>IF(B40="","",B40-C40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14">
+        <f>SUMIF($D$48:$D$147,$A41,$E$48:$E$147)</f>
+        <v/>
+      </c>
+      <c r="D41" s="14">
+        <f>IF(B41="","",B41-C41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
           <t>Contingency</t>
         </is>
       </c>
-      <c r="B36" s="14">
-        <f>SUM(B28:B35)*$B$9</f>
-        <v/>
-      </c>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14">
-        <f>B36-C36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
+      <c r="B42" s="14">
+        <f>SUM(B31:B41)*$B$9</f>
+        <v/>
+      </c>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14">
+        <f>B42-C42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B37" s="34">
-        <f>SUM(B28:B36)</f>
-        <v/>
-      </c>
-      <c r="C37" s="34">
-        <f>SUM(C28:C36)</f>
-        <v/>
-      </c>
-      <c r="D37" s="34">
-        <f>B37-C37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>The Actual total (C37) is what feeds the Basis Tracker.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="B43" s="34">
+        <f>SUM(B31:B42)</f>
+        <v/>
+      </c>
+      <c r="C43" s="34">
+        <f>SUM(C31:C42)</f>
+        <v/>
+      </c>
+      <c r="D43" s="34">
+        <f>B43-C43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>The Actual total (C43) is what feeds the Basis Tracker. Log receipts net of discount, or log the discount as a negative amount under 'Contractor discount'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>STEP 3 — COST LOG  (record every payment; Actuals above update automatically)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C47" s="9" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D47" s="9" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E47" s="9" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Payment method</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G47" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="n"/>
-      <c r="B42" s="12" t="n"/>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12" t="n"/>
-      <c r="E42" s="14" t="n"/>
-      <c r="F42" s="12" t="n"/>
-      <c r="G42" s="12" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="12" t="n"/>
-      <c r="D43" s="12" t="n"/>
-      <c r="E43" s="14" t="n"/>
-      <c r="F43" s="12" t="n"/>
-      <c r="G43" s="12" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="n"/>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="14" t="n"/>
-      <c r="F44" s="12" t="n"/>
-      <c r="G44" s="12" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n"/>
-      <c r="B45" s="12" t="n"/>
-      <c r="C45" s="12" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="12" t="n"/>
-      <c r="G45" s="12" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="n"/>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="14" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="n"/>
-      <c r="B47" s="12" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
@@ -4204,21 +4388,85 @@
       <c r="F140" s="12" t="n"/>
       <c r="G140" s="12" t="n"/>
     </row>
+    <row r="141">
+      <c r="A141" s="8" t="n"/>
+      <c r="B141" s="12" t="n"/>
+      <c r="C141" s="12" t="n"/>
+      <c r="D141" s="12" t="n"/>
+      <c r="E141" s="14" t="n"/>
+      <c r="F141" s="12" t="n"/>
+      <c r="G141" s="12" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="8" t="n"/>
+      <c r="B142" s="12" t="n"/>
+      <c r="C142" s="12" t="n"/>
+      <c r="D142" s="12" t="n"/>
+      <c r="E142" s="14" t="n"/>
+      <c r="F142" s="12" t="n"/>
+      <c r="G142" s="12" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="8" t="n"/>
+      <c r="B143" s="12" t="n"/>
+      <c r="C143" s="12" t="n"/>
+      <c r="D143" s="12" t="n"/>
+      <c r="E143" s="14" t="n"/>
+      <c r="F143" s="12" t="n"/>
+      <c r="G143" s="12" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="8" t="n"/>
+      <c r="B144" s="12" t="n"/>
+      <c r="C144" s="12" t="n"/>
+      <c r="D144" s="12" t="n"/>
+      <c r="E144" s="14" t="n"/>
+      <c r="F144" s="12" t="n"/>
+      <c r="G144" s="12" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="8" t="n"/>
+      <c r="B145" s="12" t="n"/>
+      <c r="C145" s="12" t="n"/>
+      <c r="D145" s="12" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="12" t="n"/>
+      <c r="G145" s="12" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="8" t="n"/>
+      <c r="B146" s="12" t="n"/>
+      <c r="C146" s="12" t="n"/>
+      <c r="D146" s="12" t="n"/>
+      <c r="E146" s="14" t="n"/>
+      <c r="F146" s="12" t="n"/>
+      <c r="G146" s="12" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="8" t="n"/>
+      <c r="B147" s="12" t="n"/>
+      <c r="C147" s="12" t="n"/>
+      <c r="D147" s="12" t="n"/>
+      <c r="E147" s="14" t="n"/>
+      <c r="F147" s="12" t="n"/>
+      <c r="G147" s="12" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="E19:G19"/>
     <mergeCell ref="B10:F10"/>
-    <mergeCell ref="E23:G23"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="E26:G26"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A29:G29"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>
+    <mergeCell ref="A46:G46"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4227,8 +4475,8 @@
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=$B$13:$D$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=$A$28:$A$35</formula1>
+    <dataValidation sqref="D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=$A$31:$A$41</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Strip workflow narration from workbook tabs
Section headers reduced to plain labels (OPTION COMPARISON, BUDGET vs.
ACTUAL, COST LOG, ACQUISITION COSTS, CAPITAL IMPROVEMENTS); removed
embedded how-to notes, hint text, and the template tab's usage subtitle.
Usage instructions remain only on the Read Me tab.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KP5NvhWhWoi9eWvxEnz5vK
</commit_message>
<xml_diff>
--- a/4-Indian-Brook-House-Tracker.xlsx
+++ b/4-Indian-Brook-House-Tracker.xlsx
@@ -192,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -222,7 +222,6 @@
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -735,7 +734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -790,7 +789,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>1 — ACQUISITION COSTS  (purchase price + closing costs added to basis)</t>
+          <t>ACQUISITION COSTS</t>
         </is>
       </c>
     </row>
@@ -835,11 +834,7 @@
         </is>
       </c>
       <c r="B11" s="14" t="n"/>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>From the closing disclosure</t>
-        </is>
-      </c>
+      <c r="C11" s="13" t="inlineStr"/>
       <c r="D11" s="10" t="n"/>
       <c r="E11" s="10" t="n"/>
       <c r="F11" s="11" t="n"/>
@@ -887,11 +882,7 @@
         </is>
       </c>
       <c r="B15" s="14" t="n"/>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>In MA the seller usually pays deed stamps</t>
-        </is>
-      </c>
+      <c r="C15" s="13" t="inlineStr"/>
       <c r="D15" s="10" t="n"/>
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="11" t="n"/>
@@ -922,7 +913,7 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>2 — CAPITAL IMPROVEMENTS  (auto-fed from each project tab's Actual total)</t>
+          <t>CAPITAL IMPROVEMENTS</t>
         </is>
       </c>
     </row>
@@ -1131,39 +1122,15 @@
       </c>
       <c r="E43" s="11" t="n"/>
     </row>
-    <row r="45">
-      <c r="A45" s="19" t="inlineStr">
-        <is>
-          <t>• Only capital improvements (things that add value or extend the property's life) add to basis — new floors yes, repainting a room no.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="19" t="inlineStr">
-        <is>
-          <t>• Set Capital? to N for repairs you still want to track; they'll be listed but excluded from the basis total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="19" t="inlineStr">
-        <is>
-          <t>• Keep receipts and contracts for everything on this sheet. This is a tracking aid, not tax advice.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="15">
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="D43:E43"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C12:F12"/>
-    <mergeCell ref="A45:F45"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="C15:F15"/>
@@ -1228,7 +1195,7 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Quoting</t>
         </is>
@@ -1240,7 +1207,7 @@
           <t>Contractor / quote</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>Footprints Floors of Central MA (ACS Custom Solutions Inc.) — Proposal #25584, 6/30/2026. Labor only; 50% deposit ($4,528.80) before work, balance on completion.</t>
         </is>
@@ -1252,7 +1219,7 @@
           <t>Materials source</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Floor &amp; Decor, Waltham MA (cart re-priced 7/2026); 5% materials discount through flooring contractor</t>
         </is>
@@ -1264,7 +1231,7 @@
           <t>Selected option</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n"/>
+      <c r="B8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1272,7 +1239,7 @@
           <t>Contingency %</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="21" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -1282,7 +1249,7 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Labor quote excludes materials. Subfloor leveling/remediation not included and may add cost once carpet is removed. 3% fee on credit card payments (max $3,000/card per project).</t>
         </is>
@@ -1291,7 +1258,7 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>STEP 1 — COMPARE OPTIONS  (estimated all-in cost per option)</t>
+          <t>OPTION COMPARISON</t>
         </is>
       </c>
     </row>
@@ -1301,17 +1268,17 @@
           <t>Cost component</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Sapelo Shore</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Big Sur</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Gunstock Oak</t>
         </is>
@@ -1323,27 +1290,27 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Item # / SKU</t>
         </is>
       </c>
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>101128890</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>101069698</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="D14" s="25" t="inlineStr">
         <is>
           <t>101068104</t>
         </is>
       </c>
-      <c r="E14" s="27" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>All Floor &amp; Decor. Sapelo Shore &amp; Big Sur: waterproof hybrid resilient plank w/ cork pad, 8mm 7"x51". Gunstock Oak: waterproof rigid core LVP.</t>
         </is>
@@ -1352,104 +1319,104 @@
       <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Price per box</t>
         </is>
       </c>
-      <c r="B15" s="28" t="n">
+      <c r="B15" s="27" t="n">
         <v>61.71</v>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="27" t="n">
         <v>97.08</v>
       </c>
-      <c r="D15" s="28" t="n">
+      <c r="D15" s="27" t="n">
         <v>75.56999999999999</v>
       </c>
       <c r="E15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>Boxes needed</t>
         </is>
       </c>
-      <c r="B16" s="29" t="n">
+      <c r="B16" s="28" t="n">
         <v>66</v>
       </c>
-      <c r="C16" s="29" t="n">
+      <c r="C16" s="28" t="n">
         <v>60</v>
       </c>
-      <c r="D16" s="29" t="n">
+      <c r="D16" s="28" t="n">
         <v>64</v>
       </c>
       <c r="E16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Flooring material</t>
         </is>
       </c>
-      <c r="B17" s="28">
+      <c r="B17" s="27">
         <f>B15*B16</f>
         <v/>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="27">
         <f>C15*C16</f>
         <v/>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="27">
         <f>D15*D16</f>
         <v/>
       </c>
       <c r="E17" s="12" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Underlayment &amp; supplies</t>
         </is>
       </c>
-      <c r="B18" s="28">
+      <c r="B18" s="27">
         <f>13*59.99</f>
         <v/>
       </c>
-      <c r="C18" s="28">
+      <c r="C18" s="27">
         <f>13*59.99</f>
         <v/>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="27">
         <f>13*59.99</f>
         <v/>
       </c>
-      <c r="E18" s="27" t="inlineStr">
-        <is>
-          <t>Sentinel Protect Plus underlayment — 13 rolls x $59.99 (100 sqft each), same for every option.</t>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Sentinel Protect Plus underlayment — 13 rolls x $59.99 (100 sqft each).</t>
         </is>
       </c>
       <c r="F18" s="10" t="n"/>
       <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>Stair nose trim</t>
         </is>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="27">
         <f>7*29.99</f>
         <v/>
       </c>
-      <c r="C19" s="28">
+      <c r="C19" s="27">
         <f>7*29.99</f>
         <v/>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="27">
         <f>7*29.99</f>
         <v/>
       </c>
-      <c r="E19" s="27" t="inlineStr">
+      <c r="E19" s="26" t="inlineStr">
         <is>
           <t>7 stair noses x $29.99.</t>
         </is>
@@ -1458,24 +1425,24 @@
       <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Stair risers</t>
         </is>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="27">
         <f>13*20</f>
         <v/>
       </c>
-      <c r="C20" s="28">
+      <c r="C20" s="27">
         <f>13*20</f>
         <v/>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="27">
         <f>13*20</f>
         <v/>
       </c>
-      <c r="E20" s="27" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>13 risers x $20.00.</t>
         </is>
@@ -1484,24 +1451,24 @@
       <c r="G20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Contractor discount on materials (5%)</t>
         </is>
       </c>
-      <c r="B21" s="28">
+      <c r="B21" s="27">
         <f>-0.05*SUM(B17:B20)</f>
         <v/>
       </c>
-      <c r="C21" s="28">
+      <c r="C21" s="27">
         <f>-0.05*SUM(C17:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="27">
         <f>-0.05*SUM(D17:D20)</f>
         <v/>
       </c>
-      <c r="E21" s="27" t="inlineStr">
+      <c r="E21" s="26" t="inlineStr">
         <is>
           <t>5% off all materials through the flooring contractor.</t>
         </is>
@@ -1510,41 +1477,41 @@
       <c r="G21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Est. sales tax (6.25% MA, materials)</t>
         </is>
       </c>
-      <c r="B22" s="28">
+      <c r="B22" s="27">
         <f>SUM(B17:B21)*0.0625</f>
         <v/>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="27">
         <f>SUM(C17:C21)*0.0625</f>
         <v/>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="27">
         <f>SUM(D17:D21)*0.0625</f>
         <v/>
       </c>
       <c r="E22" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Labor — demo &amp; disposal</t>
         </is>
       </c>
-      <c r="B23" s="28" t="n">
+      <c r="B23" s="27" t="n">
         <v>2642.3</v>
       </c>
-      <c r="C23" s="28" t="n">
+      <c r="C23" s="27" t="n">
         <v>2642.3</v>
       </c>
-      <c r="D23" s="28" t="n">
+      <c r="D23" s="27" t="n">
         <v>2642.3</v>
       </c>
-      <c r="E23" s="27" t="inlineStr">
+      <c r="E23" s="26" t="inlineStr">
         <is>
           <t>Footprints: demo carpet, remove &amp; return baseboards, trash removal.</t>
         </is>
@@ -1553,21 +1520,21 @@
       <c r="G23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Labor — install</t>
         </is>
       </c>
-      <c r="B24" s="28" t="n">
+      <c r="B24" s="27" t="n">
         <v>4535.3</v>
       </c>
-      <c r="C24" s="28" t="n">
+      <c r="C24" s="27" t="n">
         <v>4535.3</v>
       </c>
-      <c r="D24" s="28" t="n">
+      <c r="D24" s="27" t="n">
         <v>4535.3</v>
       </c>
-      <c r="E24" s="27" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>Footprints: install click-lock floating floor.</t>
         </is>
@@ -1576,63 +1543,57 @@
       <c r="G24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="24" t="inlineStr">
         <is>
           <t>Labor — stairs (treads &amp; risers)</t>
         </is>
       </c>
-      <c r="B25" s="28" t="n">
+      <c r="B25" s="27" t="n">
         <v>1880</v>
       </c>
-      <c r="C25" s="28" t="n">
+      <c r="C25" s="27" t="n">
         <v>1880</v>
       </c>
-      <c r="D25" s="28" t="n">
+      <c r="D25" s="27" t="n">
         <v>1880</v>
       </c>
       <c r="E25" s="12" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="30" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED</t>
         </is>
       </c>
-      <c r="B26" s="31">
+      <c r="B26" s="30">
         <f>SUM(B17:B25)</f>
         <v/>
       </c>
-      <c r="C26" s="31">
+      <c r="C26" s="30">
         <f>SUM(C17:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="30">
         <f>SUM(D17:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="27" t="inlineStr">
-        <is>
-          <t>Labor $9,057.60 is identical across options, so the spread comes entirely from the plank you pick.</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="11" t="n"/>
+      <c r="E26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>Premium vs. cheapest option</t>
         </is>
       </c>
-      <c r="B27" s="33">
+      <c r="B27" s="32">
         <f>B26-MIN($B$26:$D$26)</f>
         <v/>
       </c>
-      <c r="C27" s="33">
+      <c r="C27" s="32">
         <f>C26-MIN($B$26:$D$26)</f>
         <v/>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="32">
         <f>D26-MIN($B$26:$D$26)</f>
         <v/>
       </c>
@@ -1641,7 +1602,7 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>STEP 2 — BUDGET vs. ACTUAL  (budget auto-fills from the selected option)</t>
+          <t>BUDGET vs. ACTUAL</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1619,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Actual (from cost log)</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -1887,35 +1848,28 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="30" t="inlineStr">
+      <c r="A43" s="29" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B43" s="34">
+      <c r="B43" s="33">
         <f>SUM(B31:B42)</f>
         <v/>
       </c>
-      <c r="C43" s="34">
+      <c r="C43" s="33">
         <f>SUM(C31:C42)</f>
         <v/>
       </c>
-      <c r="D43" s="34">
+      <c r="D43" s="33">
         <f>B43-C43</f>
         <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>The Actual total (C43) is what feeds the Basis Tracker. Log receipts net of discount, or log the discount as a negative amount under 'Contractor discount'.</t>
-        </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>STEP 3 — COST LOG  (record every payment; Actuals above update automatically)</t>
+          <t>COST LOG</t>
         </is>
       </c>
     </row>
@@ -2857,12 +2811,11 @@
       <c r="G147" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A29:G29"/>
-    <mergeCell ref="E26:G26"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B10:F10"/>
@@ -2916,16 +2869,12 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PROJECT TEMPLATE — (duplicate this tab for each new project)</t>
+          <t>PROJECT TEMPLATE</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>How to use: right-click the tab &gt; Duplicate. Rename it, fill in options &amp; quotes, then add one row for it in the Basis Tracker improvements table pointing at the new tab's Actual total (cell C43).</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -2940,7 +2889,7 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
@@ -2952,7 +2901,7 @@
           <t>Contractor / quote</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr"/>
+      <c r="B6" s="19" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2960,7 +2909,7 @@
           <t>Materials source</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr"/>
+      <c r="B7" s="19" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2968,7 +2917,7 @@
           <t>Selected option</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n"/>
+      <c r="B8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2976,7 +2925,7 @@
           <t>Contingency %</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="21" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -2986,12 +2935,12 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr"/>
+      <c r="B10" s="22" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>STEP 1 — COMPARE OPTIONS  (estimated all-in cost per option)</t>
+          <t>OPTION COMPARISON</t>
         </is>
       </c>
     </row>
@@ -3001,17 +2950,17 @@
           <t>Cost component</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>Option A</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Option B</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>Option C</t>
         </is>
@@ -3023,211 +2972,199 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Item # / SKU</t>
         </is>
       </c>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-      <c r="D14" s="26" t="n"/>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n"/>
       <c r="E14" s="12" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Unit price</t>
         </is>
       </c>
-      <c r="B15" s="28" t="n"/>
-      <c r="C15" s="28" t="n"/>
-      <c r="D15" s="28" t="n"/>
+      <c r="B15" s="27" t="n"/>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="27" t="n"/>
       <c r="E15" s="12" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B16" s="29" t="n"/>
-      <c r="C16" s="29" t="n"/>
-      <c r="D16" s="29" t="n"/>
+      <c r="B16" s="28" t="n"/>
+      <c r="C16" s="28" t="n"/>
+      <c r="D16" s="28" t="n"/>
       <c r="E16" s="12" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Flooring material</t>
         </is>
       </c>
-      <c r="B17" s="28">
+      <c r="B17" s="27">
         <f>B15*B16</f>
         <v/>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="27">
         <f>C15*C16</f>
         <v/>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="27">
         <f>D15*D16</f>
         <v/>
       </c>
       <c r="E17" s="12" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Underlayment &amp; supplies</t>
         </is>
       </c>
-      <c r="B18" s="28" t="inlineStr"/>
-      <c r="C18" s="28" t="inlineStr"/>
-      <c r="D18" s="28" t="inlineStr"/>
+      <c r="B18" s="27" t="inlineStr"/>
+      <c r="C18" s="27" t="inlineStr"/>
+      <c r="D18" s="27" t="inlineStr"/>
       <c r="E18" s="12" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>Stair nose trim</t>
         </is>
       </c>
-      <c r="B19" s="28" t="inlineStr"/>
-      <c r="C19" s="28" t="inlineStr"/>
-      <c r="D19" s="28" t="inlineStr"/>
-      <c r="E19" s="27" t="inlineStr">
-        <is>
-          <t>Rename these two rows for whatever extra materials the project needs.</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="B19" s="27" t="inlineStr"/>
+      <c r="C19" s="27" t="inlineStr"/>
+      <c r="D19" s="27" t="inlineStr"/>
+      <c r="E19" s="12" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Stair risers</t>
         </is>
       </c>
-      <c r="B20" s="28" t="inlineStr"/>
-      <c r="C20" s="28" t="inlineStr"/>
-      <c r="D20" s="28" t="inlineStr"/>
+      <c r="B20" s="27" t="inlineStr"/>
+      <c r="C20" s="27" t="inlineStr"/>
+      <c r="D20" s="27" t="inlineStr"/>
       <c r="E20" s="12" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Contractor discount on materials (0%)</t>
         </is>
       </c>
-      <c r="B21" s="28">
+      <c r="B21" s="27">
         <f>-0.0*SUM(B17:B20)</f>
         <v/>
       </c>
-      <c r="C21" s="28">
+      <c r="C21" s="27">
         <f>-0.0*SUM(C17:C20)</f>
         <v/>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="27">
         <f>-0.0*SUM(D17:D20)</f>
         <v/>
       </c>
       <c r="E21" s="12" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="25" t="inlineStr">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Est. sales tax (6.25% MA, materials)</t>
         </is>
       </c>
-      <c r="B22" s="28">
+      <c r="B22" s="27">
         <f>SUM(B17:B21)*0.0625</f>
         <v/>
       </c>
-      <c r="C22" s="28">
+      <c r="C22" s="27">
         <f>SUM(C17:C21)*0.0625</f>
         <v/>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="27">
         <f>SUM(D17:D21)*0.0625</f>
         <v/>
       </c>
       <c r="E22" s="12" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Labor — demo &amp; disposal</t>
         </is>
       </c>
-      <c r="B23" s="28" t="inlineStr"/>
-      <c r="C23" s="28" t="inlineStr"/>
-      <c r="D23" s="28" t="inlineStr"/>
+      <c r="B23" s="27" t="inlineStr"/>
+      <c r="C23" s="27" t="inlineStr"/>
+      <c r="D23" s="27" t="inlineStr"/>
       <c r="E23" s="12" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="25" t="inlineStr">
+      <c r="A24" s="24" t="inlineStr">
         <is>
           <t>Labor — install</t>
         </is>
       </c>
-      <c r="B24" s="28" t="inlineStr"/>
-      <c r="C24" s="28" t="inlineStr"/>
-      <c r="D24" s="28" t="inlineStr"/>
+      <c r="B24" s="27" t="inlineStr"/>
+      <c r="C24" s="27" t="inlineStr"/>
+      <c r="D24" s="27" t="inlineStr"/>
       <c r="E24" s="12" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="24" t="inlineStr">
         <is>
           <t>Labor — stairs (treads &amp; risers)</t>
         </is>
       </c>
-      <c r="B25" s="28" t="inlineStr"/>
-      <c r="C25" s="28" t="inlineStr"/>
-      <c r="D25" s="28" t="inlineStr"/>
+      <c r="B25" s="27" t="inlineStr"/>
+      <c r="C25" s="27" t="inlineStr"/>
+      <c r="D25" s="27" t="inlineStr"/>
       <c r="E25" s="12" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="30" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED</t>
         </is>
       </c>
-      <c r="B26" s="31">
+      <c r="B26" s="30">
         <f>SUM(B17:B25)</f>
         <v/>
       </c>
-      <c r="C26" s="31">
+      <c r="C26" s="30">
         <f>SUM(C17:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="30">
         <f>SUM(D17:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="27" t="inlineStr">
-        <is>
-          <t>Compare options here, pick one in 'Selected option' above, and the budget below fills itself in.</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="11" t="n"/>
+      <c r="E26" s="12" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>Premium vs. cheapest option</t>
         </is>
       </c>
-      <c r="B27" s="33">
+      <c r="B27" s="32">
         <f>B26-MIN($B$26:$D$26)</f>
         <v/>
       </c>
-      <c r="C27" s="33">
+      <c r="C27" s="32">
         <f>C26-MIN($B$26:$D$26)</f>
         <v/>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="32">
         <f>D26-MIN($B$26:$D$26)</f>
         <v/>
       </c>
@@ -3236,7 +3173,7 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>STEP 2 — BUDGET vs. ACTUAL  (budget auto-fills from the selected option)</t>
+          <t>BUDGET vs. ACTUAL</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3190,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Actual (from cost log)</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -3482,35 +3419,28 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="30" t="inlineStr">
+      <c r="A43" s="29" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B43" s="34">
+      <c r="B43" s="33">
         <f>SUM(B31:B42)</f>
         <v/>
       </c>
-      <c r="C43" s="34">
+      <c r="C43" s="33">
         <f>SUM(C31:C42)</f>
         <v/>
       </c>
-      <c r="D43" s="34">
+      <c r="D43" s="33">
         <f>B43-C43</f>
         <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>The Actual total (C43) is what feeds the Basis Tracker. Log receipts net of discount, or log the discount as a negative amount under 'Contractor discount'.</t>
-        </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>STEP 3 — COST LOG  (record every payment; Actuals above update automatically)</t>
+          <t>COST LOG</t>
         </is>
       </c>
     </row>
@@ -4452,16 +4382,14 @@
       <c r="G147" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="12">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="E19:G19"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="E26:G26"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="B8:F8"/>

</xml_diff>

<commit_message>
Add homeowner reference tabs and fix estimate double-counting
- Project Estimates: new Count? (Y/N) column; totals use SUMIFS so
  competing quotes for the same project stay listed without inflating
  the totals
- Vendors & Contacts: directory seeded with Footprints Floors and
  Floor & Decor
- Finishes & Materials: room-by-room record of paint/flooring/fixture
  SKUs, seeded with the 2nd-floor LVP row
- Appliances & Systems: 19 pre-seeded items with typical lifespan and
  service cadence; suggested replacement date computes from install
  date + lifespan (blank until dates are entered)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KP5NvhWhWoi9eWvxEnz5vK
</commit_message>
<xml_diff>
--- a/4-Indian-Brook-House-Tracker.xlsx
+++ b/4-Indian-Brook-House-Tracker.xlsx
@@ -11,7 +11,10 @@
     <sheet name="2nd Floor Flooring" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Project Estimates" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Project Template" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Read Me" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Vendors &amp; Contacts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Finishes &amp; Materials" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Appliances &amp; Systems" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Read Me" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -193,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -256,6 +259,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -2746,7 +2752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2755,7 +2761,8 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2775,22 +2782,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Total estimated — all</t>
+          <t>Total estimated — counted quotes</t>
         </is>
       </c>
       <c r="B4" s="12">
-        <f>SUM(E9:E58)</f>
+        <f>SUMIFS(E9:E58,G9:G58,"Y")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Total estimated — marked Now</t>
+          <t>Total estimated — counted &amp; marked Now</t>
         </is>
       </c>
       <c r="B5" s="12">
-        <f>SUMIF(F9:F58,"Now",E9:E58)</f>
+        <f>SUMIFS(E9:E58,G9:G58,"Y",F9:F58,"Now")</f>
         <v/>
       </c>
     </row>
@@ -2833,6 +2840,11 @@
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Count?</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2853,7 +2865,12 @@
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="12" t="n"/>
       <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -2870,7 +2887,12 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="12" t="n"/>
       <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>
@@ -2879,7 +2901,8 @@
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="12" t="n"/>
       <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="10" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n"/>
@@ -2888,7 +2911,8 @@
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="12" t="n"/>
       <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="10" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n"/>
@@ -2897,7 +2921,8 @@
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="12" t="n"/>
       <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="10" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -2906,7 +2931,8 @@
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="12" t="n"/>
       <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="G14" s="23" t="n"/>
+      <c r="H14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n"/>
@@ -2915,7 +2941,8 @@
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="12" t="n"/>
       <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="10" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -2924,7 +2951,8 @@
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="12" t="n"/>
       <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="G16" s="23" t="n"/>
+      <c r="H16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -2933,7 +2961,8 @@
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="12" t="n"/>
       <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -2942,7 +2971,8 @@
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="12" t="n"/>
       <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="G18" s="23" t="n"/>
+      <c r="H18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n"/>
@@ -2951,7 +2981,8 @@
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="12" t="n"/>
       <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="G19" s="23" t="n"/>
+      <c r="H19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -2960,7 +2991,8 @@
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="12" t="n"/>
       <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="G20" s="23" t="n"/>
+      <c r="H20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n"/>
@@ -2969,7 +3001,8 @@
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="12" t="n"/>
       <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
+      <c r="G21" s="23" t="n"/>
+      <c r="H21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -2978,7 +3011,8 @@
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="12" t="n"/>
       <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -2987,7 +3021,8 @@
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="12" t="n"/>
       <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -2996,7 +3031,8 @@
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="12" t="n"/>
       <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
+      <c r="G24" s="23" t="n"/>
+      <c r="H24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n"/>
@@ -3005,7 +3041,8 @@
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="12" t="n"/>
       <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -3014,7 +3051,8 @@
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="12" t="n"/>
       <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n"/>
@@ -3023,7 +3061,8 @@
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="12" t="n"/>
       <c r="F27" s="10" t="n"/>
-      <c r="G27" s="10" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -3032,7 +3071,8 @@
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="12" t="n"/>
       <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n"/>
@@ -3041,7 +3081,8 @@
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="12" t="n"/>
       <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="H29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -3050,7 +3091,8 @@
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="12" t="n"/>
       <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n"/>
@@ -3059,7 +3101,8 @@
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="12" t="n"/>
       <c r="F31" s="10" t="n"/>
-      <c r="G31" s="10" t="n"/>
+      <c r="G31" s="23" t="n"/>
+      <c r="H31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -3068,7 +3111,8 @@
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="12" t="n"/>
       <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="10" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -3077,7 +3121,8 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="12" t="n"/>
       <c r="F33" s="10" t="n"/>
-      <c r="G33" s="10" t="n"/>
+      <c r="G33" s="23" t="n"/>
+      <c r="H33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -3086,7 +3131,8 @@
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="12" t="n"/>
       <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
+      <c r="G34" s="23" t="n"/>
+      <c r="H34" s="10" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n"/>
@@ -3095,7 +3141,8 @@
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="12" t="n"/>
       <c r="F35" s="10" t="n"/>
-      <c r="G35" s="10" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="10" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -3104,7 +3151,8 @@
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="12" t="n"/>
       <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
+      <c r="G36" s="23" t="n"/>
+      <c r="H36" s="10" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n"/>
@@ -3113,7 +3161,8 @@
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="12" t="n"/>
       <c r="F37" s="10" t="n"/>
-      <c r="G37" s="10" t="n"/>
+      <c r="G37" s="23" t="n"/>
+      <c r="H37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -3122,7 +3171,8 @@
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="12" t="n"/>
       <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
+      <c r="G38" s="23" t="n"/>
+      <c r="H38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n"/>
@@ -3131,7 +3181,8 @@
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="12" t="n"/>
       <c r="F39" s="10" t="n"/>
-      <c r="G39" s="10" t="n"/>
+      <c r="G39" s="23" t="n"/>
+      <c r="H39" s="10" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -3140,7 +3191,8 @@
       <c r="D40" s="6" t="n"/>
       <c r="E40" s="12" t="n"/>
       <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
+      <c r="G40" s="23" t="n"/>
+      <c r="H40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n"/>
@@ -3149,7 +3201,8 @@
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="12" t="n"/>
       <c r="F41" s="10" t="n"/>
-      <c r="G41" s="10" t="n"/>
+      <c r="G41" s="23" t="n"/>
+      <c r="H41" s="10" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -3158,7 +3211,8 @@
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="12" t="n"/>
       <c r="F42" s="10" t="n"/>
-      <c r="G42" s="10" t="n"/>
+      <c r="G42" s="23" t="n"/>
+      <c r="H42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n"/>
@@ -3167,7 +3221,8 @@
       <c r="D43" s="6" t="n"/>
       <c r="E43" s="12" t="n"/>
       <c r="F43" s="10" t="n"/>
-      <c r="G43" s="10" t="n"/>
+      <c r="G43" s="23" t="n"/>
+      <c r="H43" s="10" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -3176,7 +3231,8 @@
       <c r="D44" s="6" t="n"/>
       <c r="E44" s="12" t="n"/>
       <c r="F44" s="10" t="n"/>
-      <c r="G44" s="10" t="n"/>
+      <c r="G44" s="23" t="n"/>
+      <c r="H44" s="10" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n"/>
@@ -3185,7 +3241,8 @@
       <c r="D45" s="6" t="n"/>
       <c r="E45" s="12" t="n"/>
       <c r="F45" s="10" t="n"/>
-      <c r="G45" s="10" t="n"/>
+      <c r="G45" s="23" t="n"/>
+      <c r="H45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -3194,7 +3251,8 @@
       <c r="D46" s="6" t="n"/>
       <c r="E46" s="12" t="n"/>
       <c r="F46" s="10" t="n"/>
-      <c r="G46" s="10" t="n"/>
+      <c r="G46" s="23" t="n"/>
+      <c r="H46" s="10" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n"/>
@@ -3203,7 +3261,8 @@
       <c r="D47" s="6" t="n"/>
       <c r="E47" s="12" t="n"/>
       <c r="F47" s="10" t="n"/>
-      <c r="G47" s="10" t="n"/>
+      <c r="G47" s="23" t="n"/>
+      <c r="H47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -3212,7 +3271,8 @@
       <c r="D48" s="6" t="n"/>
       <c r="E48" s="12" t="n"/>
       <c r="F48" s="10" t="n"/>
-      <c r="G48" s="10" t="n"/>
+      <c r="G48" s="23" t="n"/>
+      <c r="H48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n"/>
@@ -3221,7 +3281,8 @@
       <c r="D49" s="6" t="n"/>
       <c r="E49" s="12" t="n"/>
       <c r="F49" s="10" t="n"/>
-      <c r="G49" s="10" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="H49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -3230,7 +3291,8 @@
       <c r="D50" s="6" t="n"/>
       <c r="E50" s="12" t="n"/>
       <c r="F50" s="10" t="n"/>
-      <c r="G50" s="10" t="n"/>
+      <c r="G50" s="23" t="n"/>
+      <c r="H50" s="10" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n"/>
@@ -3239,7 +3301,8 @@
       <c r="D51" s="6" t="n"/>
       <c r="E51" s="12" t="n"/>
       <c r="F51" s="10" t="n"/>
-      <c r="G51" s="10" t="n"/>
+      <c r="G51" s="23" t="n"/>
+      <c r="H51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -3248,7 +3311,8 @@
       <c r="D52" s="6" t="n"/>
       <c r="E52" s="12" t="n"/>
       <c r="F52" s="10" t="n"/>
-      <c r="G52" s="10" t="n"/>
+      <c r="G52" s="23" t="n"/>
+      <c r="H52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n"/>
@@ -3257,7 +3321,8 @@
       <c r="D53" s="6" t="n"/>
       <c r="E53" s="12" t="n"/>
       <c r="F53" s="10" t="n"/>
-      <c r="G53" s="10" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="H53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -3266,7 +3331,8 @@
       <c r="D54" s="6" t="n"/>
       <c r="E54" s="12" t="n"/>
       <c r="F54" s="10" t="n"/>
-      <c r="G54" s="10" t="n"/>
+      <c r="G54" s="23" t="n"/>
+      <c r="H54" s="10" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n"/>
@@ -3275,7 +3341,8 @@
       <c r="D55" s="6" t="n"/>
       <c r="E55" s="12" t="n"/>
       <c r="F55" s="10" t="n"/>
-      <c r="G55" s="10" t="n"/>
+      <c r="G55" s="23" t="n"/>
+      <c r="H55" s="10" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -3284,7 +3351,8 @@
       <c r="D56" s="6" t="n"/>
       <c r="E56" s="12" t="n"/>
       <c r="F56" s="10" t="n"/>
-      <c r="G56" s="10" t="n"/>
+      <c r="G56" s="23" t="n"/>
+      <c r="H56" s="10" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="n"/>
@@ -3293,7 +3361,8 @@
       <c r="D57" s="6" t="n"/>
       <c r="E57" s="12" t="n"/>
       <c r="F57" s="10" t="n"/>
-      <c r="G57" s="10" t="n"/>
+      <c r="G57" s="23" t="n"/>
+      <c r="H57" s="10" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -3302,17 +3371,21 @@
       <c r="D58" s="6" t="n"/>
       <c r="E58" s="12" t="n"/>
       <c r="F58" s="10" t="n"/>
-      <c r="G58" s="10" t="n"/>
+      <c r="G58" s="23" t="n"/>
+      <c r="H58" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 F21 F22 F23 F24 F25 F26 F27 F28 F29 F30 F31 F32 F33 F34 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44 F45 F46 F47 F48 F49 F50 F51 F52 F53 F54 F55 F56 F57 F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Now,Later,Undecided,Passed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51 G52 G53 G54 G55 G56 G57 G58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4886,11 +4959,1999 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>VENDORS &amp; CONTACTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>4 Indian Brook Road, Ashland, MA 01721</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DIRECTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Trade / service</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Used for</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Use again?</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Footprints Floors of Central MA</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Flooring install</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>S. Donohoe</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>(508) 422-4545</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>sdonohoe@footprintsfloors.com</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>2nd floor flooring</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="n"/>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>ACS Custom Solutions Inc.; proposal #25584</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Floor &amp; Decor — Waltham</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Flooring materials</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>2nd floor flooring materials</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="n"/>
+      <c r="H7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="23" t="n"/>
+      <c r="H9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="23" t="n"/>
+      <c r="H10" s="10" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="23" t="n"/>
+      <c r="H13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="23" t="n"/>
+      <c r="H14" s="10" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="23" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="23" t="n"/>
+      <c r="H16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="23" t="n"/>
+      <c r="H18" s="10" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="23" t="n"/>
+      <c r="H19" s="10" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="23" t="n"/>
+      <c r="H20" s="10" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="23" t="n"/>
+      <c r="H21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="23" t="n"/>
+      <c r="H22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="23" t="n"/>
+      <c r="H23" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="23" t="n"/>
+      <c r="H24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="10" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="H29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="10" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="23" t="n"/>
+      <c r="H31" s="10" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="23" t="n"/>
+      <c r="H33" s="10" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="23" t="n"/>
+      <c r="H34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="10" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="23" t="n"/>
+      <c r="H36" s="10" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="23" t="n"/>
+      <c r="H37" s="10" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="23" t="n"/>
+      <c r="H38" s="10" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="10" t="n"/>
+      <c r="G39" s="23" t="n"/>
+      <c r="H39" s="10" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n"/>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="23" t="n"/>
+      <c r="H40" s="10" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n"/>
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="10" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="23" t="n"/>
+      <c r="H41" s="10" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n"/>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="23" t="n"/>
+      <c r="H42" s="10" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="n"/>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="10" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="23" t="n"/>
+      <c r="H43" s="10" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="10" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="23" t="n"/>
+      <c r="H44" s="10" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n"/>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="10" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="23" t="n"/>
+      <c r="H45" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FINISHES &amp; MATERIALS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>4 Indian Brook Road, Ashland, MA 01721</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>RECORD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Room / area</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Brand / product</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Color / finish</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>SKU / code</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Where purchased</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Second floor</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Flooring — LVP</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Floor &amp; Decor — Waltham</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="10" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="10" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="10" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="10" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="10" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="10" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="10" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="10" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="10" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="10" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="10" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="10" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="10" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="10" t="n"/>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="10" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n"/>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="10" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n"/>
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="10" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="10" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n"/>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="10" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="n"/>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="10" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="10" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="10" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="10" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n"/>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="10" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="10" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="10" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="n"/>
+      <c r="D47" s="10" t="n"/>
+      <c r="E47" s="10" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="10" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="n"/>
+      <c r="B48" s="10" t="n"/>
+      <c r="C48" s="10" t="n"/>
+      <c r="D48" s="10" t="n"/>
+      <c r="E48" s="10" t="n"/>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="10" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="n"/>
+      <c r="B49" s="10" t="n"/>
+      <c r="C49" s="10" t="n"/>
+      <c r="D49" s="10" t="n"/>
+      <c r="E49" s="10" t="n"/>
+      <c r="F49" s="10" t="n"/>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="10" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="n"/>
+      <c r="B50" s="10" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="10" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n"/>
+      <c r="B51" s="10" t="n"/>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="10" t="n"/>
+      <c r="E51" s="10" t="n"/>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="10" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="n"/>
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="10" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="10" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="n"/>
+      <c r="B53" s="10" t="n"/>
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="10" t="n"/>
+      <c r="E53" s="10" t="n"/>
+      <c r="F53" s="10" t="n"/>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="10" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n"/>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="10" t="n"/>
+      <c r="E54" s="10" t="n"/>
+      <c r="F54" s="10" t="n"/>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="10" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n"/>
+      <c r="B55" s="10" t="n"/>
+      <c r="C55" s="10" t="n"/>
+      <c r="D55" s="10" t="n"/>
+      <c r="E55" s="10" t="n"/>
+      <c r="F55" s="10" t="n"/>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>APPLIANCES &amp; SYSTEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>4 Indian Brook Road, Ashland, MA 01721</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>INVENTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Make &amp; model</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Serial #</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Install date</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Warranty expires</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Typical lifespan (yrs)</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Suggested replacement</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Service cadence</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Last serviced</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Heating system (furnace / boiler)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Basement</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="6">
+        <f>IF(OR(E6="",G6=""),"",EDATE(E6,12*G6))</f>
+        <v/>
+      </c>
+      <c r="I6" s="32" t="inlineStr">
+        <is>
+          <t>Annual tune-up; replace filters every 1-3 months (forced air)</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Central A/C / heat pump</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Exterior + attic</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" s="6">
+        <f>IF(OR(E7="",G7=""),"",EDATE(E7,12*G7))</f>
+        <v/>
+      </c>
+      <c r="I7" s="32" t="inlineStr">
+        <is>
+          <t>Annual tune-up; keep outdoor unit clear</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Water heater</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Basement</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="6">
+        <f>IF(OR(E8="",G8=""),"",EDATE(E8,12*G8))</f>
+        <v/>
+      </c>
+      <c r="I8" s="32" t="inlineStr">
+        <is>
+          <t>Flush tank annually; test T&amp;P valve</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Refrigerator</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="H9" s="6">
+        <f>IF(OR(E9="",G9=""),"",EDATE(E9,12*G9))</f>
+        <v/>
+      </c>
+      <c r="I9" s="32" t="inlineStr">
+        <is>
+          <t>Vacuum coils annually</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Range / oven</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="H10" s="6">
+        <f>IF(OR(E10="",G10=""),"",EDATE(E10,12*G10))</f>
+        <v/>
+      </c>
+      <c r="I10" s="32" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="10" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Dishwasher</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" s="6">
+        <f>IF(OR(E11="",G11=""),"",EDATE(E11,12*G11))</f>
+        <v/>
+      </c>
+      <c r="I11" s="32" t="inlineStr">
+        <is>
+          <t>Clean filter quarterly</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Microwave</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" s="6">
+        <f>IF(OR(E12="",G12=""),"",EDATE(E12,12*G12))</f>
+        <v/>
+      </c>
+      <c r="I12" s="32" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Washer</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Laundry</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="H13" s="6">
+        <f>IF(OR(E13="",G13=""),"",EDATE(E13,12*G13))</f>
+        <v/>
+      </c>
+      <c r="I13" s="32" t="inlineStr">
+        <is>
+          <t>Inspect supply hoses annually</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Dryer</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Laundry</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="H14" s="6">
+        <f>IF(OR(E14="",G14=""),"",EDATE(E14,12*G14))</f>
+        <v/>
+      </c>
+      <c r="I14" s="32" t="inlineStr">
+        <is>
+          <t>Clean vent duct annually; lint trap every load</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="10" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Garbage disposal</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" s="6">
+        <f>IF(OR(E15="",G15=""),"",EDATE(E15,12*G15))</f>
+        <v/>
+      </c>
+      <c r="I15" s="32" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Sump pump</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Basement</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H16" s="6">
+        <f>IF(OR(E16="",G16=""),"",EDATE(E16,12*G16))</f>
+        <v/>
+      </c>
+      <c r="I16" s="32" t="inlineStr">
+        <is>
+          <t>Test quarterly; check before spring thaw</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="n"/>
+      <c r="K16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Roof (asphalt shingle)</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Exterior</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="H17" s="6">
+        <f>IF(OR(E17="",G17=""),"",EDATE(E17,12*G17))</f>
+        <v/>
+      </c>
+      <c r="I17" s="32" t="inlineStr">
+        <is>
+          <t>Inspect annually and after major storms</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Gutters &amp; downspouts</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Exterior</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="H18" s="6">
+        <f>IF(OR(E18="",G18=""),"",EDATE(E18,12*G18))</f>
+        <v/>
+      </c>
+      <c r="I18" s="32" t="inlineStr">
+        <is>
+          <t>Clean spring and fall</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="10" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Whole house</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="H19" s="6">
+        <f>IF(OR(E19="",G19=""),"",EDATE(E19,12*G19))</f>
+        <v/>
+      </c>
+      <c r="I19" s="32" t="inlineStr">
+        <is>
+          <t>Check seals/caulk annually</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="10" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Deck / porch</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Exterior</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="H20" s="6">
+        <f>IF(OR(E20="",G20=""),"",EDATE(E20,12*G20))</f>
+        <v/>
+      </c>
+      <c r="I20" s="32" t="inlineStr">
+        <is>
+          <t>Reseal or restain every 2-3 years</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="10" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Garage door &amp; opener</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Garage</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" s="6">
+        <f>IF(OR(E21="",G21=""),"",EDATE(E21,12*G21))</f>
+        <v/>
+      </c>
+      <c r="I21" s="32" t="inlineStr">
+        <is>
+          <t>Lubricate tracks/rollers annually</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Smoke / CO detectors</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Whole house</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" s="6">
+        <f>IF(OR(E22="",G22=""),"",EDATE(E22,12*G22))</f>
+        <v/>
+      </c>
+      <c r="I22" s="32" t="inlineStr">
+        <is>
+          <t>Test monthly; replace batteries annually</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Septic system (if applicable)</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Exterior</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="H23" s="6">
+        <f>IF(OR(E23="",G23=""),"",EDATE(E23,12*G23))</f>
+        <v/>
+      </c>
+      <c r="I23" s="32" t="inlineStr">
+        <is>
+          <t>Pump every 2-3 years; Title 5 inspection at sale</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="n"/>
+      <c r="K23" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Irrigation system (if applicable)</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Exterior</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="H24" s="6">
+        <f>IF(OR(E24="",G24=""),"",EDATE(E24,12*G24))</f>
+        <v/>
+      </c>
+      <c r="I24" s="32" t="inlineStr">
+        <is>
+          <t>Winterize every fall; startup check in spring</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="6">
+        <f>IF(OR(E25="",G25=""),"",EDATE(E25,12*G25))</f>
+        <v/>
+      </c>
+      <c r="I25" s="32" t="n"/>
+      <c r="J25" s="6" t="n"/>
+      <c r="K25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="6">
+        <f>IF(OR(E26="",G26=""),"",EDATE(E26,12*G26))</f>
+        <v/>
+      </c>
+      <c r="I26" s="32" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="23" t="n"/>
+      <c r="H27" s="6">
+        <f>IF(OR(E27="",G27=""),"",EDATE(E27,12*G27))</f>
+        <v/>
+      </c>
+      <c r="I27" s="32" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="6">
+        <f>IF(OR(E28="",G28=""),"",EDATE(E28,12*G28))</f>
+        <v/>
+      </c>
+      <c r="I28" s="32" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="10" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="23" t="n"/>
+      <c r="H29" s="6">
+        <f>IF(OR(E29="",G29=""),"",EDATE(E29,12*G29))</f>
+        <v/>
+      </c>
+      <c r="I29" s="32" t="n"/>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="23" t="n"/>
+      <c r="H30" s="6">
+        <f>IF(OR(E30="",G30=""),"",EDATE(E30,12*G30))</f>
+        <v/>
+      </c>
+      <c r="I30" s="32" t="n"/>
+      <c r="J30" s="6" t="n"/>
+      <c r="K30" s="10" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="23" t="n"/>
+      <c r="H31" s="6">
+        <f>IF(OR(E31="",G31=""),"",EDATE(E31,12*G31))</f>
+        <v/>
+      </c>
+      <c r="I31" s="32" t="n"/>
+      <c r="J31" s="6" t="n"/>
+      <c r="K31" s="10" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="23" t="n"/>
+      <c r="H32" s="6">
+        <f>IF(OR(E32="",G32=""),"",EDATE(E32,12*G32))</f>
+        <v/>
+      </c>
+      <c r="I32" s="32" t="n"/>
+      <c r="J32" s="6" t="n"/>
+      <c r="K32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="23" t="n"/>
+      <c r="H33" s="6">
+        <f>IF(OR(E33="",G33=""),"",EDATE(E33,12*G33))</f>
+        <v/>
+      </c>
+      <c r="I33" s="32" t="n"/>
+      <c r="J33" s="6" t="n"/>
+      <c r="K33" s="10" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="23" t="n"/>
+      <c r="H34" s="6">
+        <f>IF(OR(E34="",G34=""),"",EDATE(E34,12*G34))</f>
+        <v/>
+      </c>
+      <c r="I34" s="32" t="n"/>
+      <c r="J34" s="6" t="n"/>
+      <c r="K34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="6">
+        <f>IF(OR(E35="",G35=""),"",EDATE(E35,12*G35))</f>
+        <v/>
+      </c>
+      <c r="I35" s="32" t="n"/>
+      <c r="J35" s="6" t="n"/>
+      <c r="K35" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A4:K4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4912,84 +6973,120 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>What this is</t>
         </is>
       </c>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B4" s="34" t="inlineStr">
         <is>
           <t>One workbook that tracks what the house cost and every project that adds to it. Share it in Google Drive so both of you can edit.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>Basis Tracker</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="34" t="inlineStr">
         <is>
           <t>Purchase price ($1,060,000, closing 7/17/2026) + closing costs + capital improvements = adjusted cost basis. Each project tab feeds one row of the improvements table.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>2nd Floor Flooring</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
+      <c r="B7" s="34" t="inlineStr">
         <is>
           <t>First project. Compare the 3 Floor &amp; Decor plank options (incl. underlayment, stair nose &amp; risers, 5% contractor discount, est. tax, and Footprints labor), pick one in 'Selected option' (yellow cell), and the budget fills in automatically. Log payments in the cost log at the bottom — actuals and the Basis Tracker update themselves.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="32" t="inlineStr">
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
         <is>
           <t>Project Estimates</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>Preliminary phase: log each quote you collect (HVAC, carpentry, etc.) with its estimated cost, and mark Timing (Now / Later / Undecided / Passed) to decide what to take on. When a project is a go, give it its own tab from the template.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>Preliminary phase: log each quote you collect (HVAC, carpentry, etc.) with its estimated cost, and mark Timing (Now / Later / Undecided / Passed) to decide what to take on. Set Count? to Y on the one quote per project you'd actually use — competing quotes marked N stay listed but don't double-count in the totals. When a project is a go, give it its own tab from the template.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Vendors &amp; Contacts</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>Directory of contractors, suppliers, and service companies used on the house.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Finishes &amp; Materials</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>Room-by-room record of paint colors, flooring, fixtures, and their SKUs — for touch-ups and matching repairs later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>Appliances &amp; Systems</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>Inventory of the house's equipment with make/model/serial, warranty dates, and service cadence. Enter an install date and the suggested replacement date computes from the typical lifespan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Project Template</t>
         </is>
       </c>
-      <c r="B9" s="33" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>For the next project: right-click the tab &gt; Duplicate, rename it, fill in your options/quotes, then add a row in the Basis Tracker improvements table pointing at the new tab's cell C43 (its Actual total).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="32" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B11" s="33" t="inlineStr">
+      <c r="B14" s="34" t="inlineStr">
         <is>
           <t>Labor: Footprints Floors of Central MA proposal #25584 (6/30/2026) — $9,057.60, materials excluded. Materials: Floor &amp; Decor Waltham cart (7/2026) — Sapelo Shore / Big Sur / Gunstock Oak + Sentinel underlayment (15 rolls), plus 7 stair noses @ $29.99 and 13 risers @ $20; 5% contractor discount on materials.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Tip</t>
         </is>
       </c>
-      <c r="B13" s="33" t="inlineStr">
+      <c r="B16" s="34" t="inlineStr">
         <is>
           <t>In Google Sheets everything here — dropdowns, cross-tab formulas, formatting — survives File &gt; Import. Use 'Replace spreadsheet' when importing so tab references stay intact.</t>
         </is>

</xml_diff>

<commit_message>
Remove underlayment line item — attached to plank, no separate order
Drops the row from the option comparison, budget, and cost-log
categories; sales tax and discount now compute on flooring + stair
parts only. Layout constants shift the Basis Tracker link to the new
Actual total cell automatically.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KP5NvhWhWoi9eWvxEnz5vK
</commit_message>
<xml_diff>
--- a/4-Indian-Brook-House-Tracker.xlsx
+++ b/4-Indian-Brook-House-Tracker.xlsx
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="E21" s="12">
-        <f>'2nd Floor Flooring'!C43</f>
+        <f>'2nd Floor Flooring'!C41</f>
         <v/>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G147"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>All Floor &amp; Decor. Sapelo Shore &amp; Big Sur: waterproof hybrid resilient plank w/ cork pad, 8mm 7"x51". Gunstock Oak: waterproof rigid core LVP.</t>
+          <t>All Floor &amp; Decor. Sapelo Shore &amp; Big Sur: waterproof hybrid resilient plank w/ cork pad, 8mm 7"x51". Gunstock Oak: waterproof rigid core LVP. Underlayment attached — no separate order.</t>
         </is>
       </c>
       <c r="F14" s="8" t="n"/>
@@ -1273,24 +1273,24 @@
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>Underlayment &amp; supplies</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B18" s="25">
-        <f>15*59.99</f>
+        <f>7*29.99</f>
         <v/>
       </c>
       <c r="C18" s="25">
-        <f>15*59.99</f>
+        <f>7*29.99</f>
         <v/>
       </c>
       <c r="D18" s="25">
-        <f>15*59.99</f>
+        <f>7*29.99</f>
         <v/>
       </c>
       <c r="E18" s="24" t="inlineStr">
         <is>
-          <t>Sentinel Protect Plus underlayment — 15 rolls x $59.99 (100 sqft each).</t>
+          <t>7 stair noses x $29.99.</t>
         </is>
       </c>
       <c r="F18" s="8" t="n"/>
@@ -1299,24 +1299,24 @@
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>Stair nose trim</t>
+          <t>Stair risers</t>
         </is>
       </c>
       <c r="B19" s="25">
-        <f>7*29.99</f>
+        <f>13*20</f>
         <v/>
       </c>
       <c r="C19" s="25">
-        <f>7*29.99</f>
+        <f>13*20</f>
         <v/>
       </c>
       <c r="D19" s="25">
-        <f>7*29.99</f>
+        <f>13*20</f>
         <v/>
       </c>
       <c r="E19" s="24" t="inlineStr">
         <is>
-          <t>7 stair noses x $29.99.</t>
+          <t>13 risers x $20.00.</t>
         </is>
       </c>
       <c r="F19" s="8" t="n"/>
@@ -1325,24 +1325,24 @@
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
         <is>
-          <t>Stair risers</t>
+          <t>Contractor discount on materials (5%)</t>
         </is>
       </c>
       <c r="B20" s="25">
-        <f>13*20</f>
+        <f>-0.05*SUM(B17:B19)</f>
         <v/>
       </c>
       <c r="C20" s="25">
-        <f>13*20</f>
+        <f>-0.05*SUM(C17:C19)</f>
         <v/>
       </c>
       <c r="D20" s="25">
-        <f>13*20</f>
+        <f>-0.05*SUM(D17:D19)</f>
         <v/>
       </c>
       <c r="E20" s="24" t="inlineStr">
         <is>
-          <t>13 risers x $20.00.</t>
+          <t>5% off all materials through the flooring contractor.</t>
         </is>
       </c>
       <c r="F20" s="8" t="n"/>
@@ -1351,67 +1351,64 @@
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
-          <t>Contractor discount on materials (5%)</t>
+          <t>Est. sales tax (6.25% MA, materials)</t>
         </is>
       </c>
       <c r="B21" s="25">
-        <f>-0.05*SUM(B17:B20)</f>
+        <f>SUM(B17:B20)*0.0625</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>-0.05*SUM(C17:C20)</f>
+        <f>SUM(C17:C20)*0.0625</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>-0.05*SUM(D17:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="24" t="inlineStr">
-        <is>
-          <t>5% off all materials through the flooring contractor.</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="9" t="n"/>
+        <f>SUM(D17:D20)*0.0625</f>
+        <v/>
+      </c>
+      <c r="E21" s="10" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>Est. sales tax (6.25% MA, materials)</t>
-        </is>
-      </c>
-      <c r="B22" s="25">
-        <f>SUM(B17:B21)*0.0625</f>
-        <v/>
-      </c>
-      <c r="C22" s="25">
-        <f>SUM(C17:C21)*0.0625</f>
-        <v/>
-      </c>
-      <c r="D22" s="25">
-        <f>SUM(D17:D21)*0.0625</f>
-        <v/>
-      </c>
-      <c r="E22" s="10" t="n"/>
+          <t>Labor — demo &amp; disposal</t>
+        </is>
+      </c>
+      <c r="B22" s="25" t="n">
+        <v>2642.3</v>
+      </c>
+      <c r="C22" s="25" t="n">
+        <v>2642.3</v>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>2642.3</v>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>Footprints: demo carpet, remove &amp; return baseboards, trash removal.</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Labor — install</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
-        <v>2642.3</v>
+        <v>4535.3</v>
       </c>
       <c r="C23" s="25" t="n">
-        <v>2642.3</v>
+        <v>4535.3</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>2642.3</v>
+        <v>4535.3</v>
       </c>
       <c r="E23" s="24" t="inlineStr">
         <is>
-          <t>Footprints: demo carpet, remove &amp; return baseboards, trash removal.</t>
+          <t>Footprints: install click-lock floating floor.</t>
         </is>
       </c>
       <c r="F23" s="8" t="n"/>
@@ -1420,124 +1417,120 @@
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>Labor — install</t>
+          <t>Labor — stairs (treads &amp; risers)</t>
         </is>
       </c>
       <c r="B24" s="25" t="n">
-        <v>4535.3</v>
+        <v>1880</v>
       </c>
       <c r="C24" s="25" t="n">
-        <v>4535.3</v>
+        <v>1880</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>4535.3</v>
-      </c>
-      <c r="E24" s="24" t="inlineStr">
-        <is>
-          <t>Footprints: install click-lock floating floor.</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="n"/>
-      <c r="G24" s="9" t="n"/>
+        <v>1880</v>
+      </c>
+      <c r="E24" s="10" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
-        <is>
-          <t>Labor — stairs (treads &amp; risers)</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="n">
-        <v>1880</v>
-      </c>
-      <c r="C25" s="25" t="n">
-        <v>1880</v>
-      </c>
-      <c r="D25" s="25" t="n">
-        <v>1880</v>
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>TOTAL ESTIMATED</t>
+        </is>
+      </c>
+      <c r="B25" s="28">
+        <f>SUM(B17:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="28">
+        <f>SUM(C17:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="28">
+        <f>SUM(D17:D24)</f>
+        <v/>
       </c>
       <c r="E25" s="10" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
-        <is>
-          <t>TOTAL ESTIMATED</t>
-        </is>
-      </c>
-      <c r="B26" s="28">
-        <f>SUM(B17:B25)</f>
-        <v/>
-      </c>
-      <c r="C26" s="28">
-        <f>SUM(C17:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="28">
-        <f>SUM(D17:D25)</f>
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Premium vs. cheapest option</t>
+        </is>
+      </c>
+      <c r="B26" s="30">
+        <f>B25-MIN($B$25:$D$25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="30">
+        <f>C25-MIN($B$25:$D$25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="30">
+        <f>D25-MIN($B$25:$D$25)</f>
         <v/>
       </c>
       <c r="E26" s="10" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="29" t="inlineStr">
-        <is>
-          <t>Premium vs. cheapest option</t>
-        </is>
-      </c>
-      <c r="B27" s="30">
-        <f>B26-MIN($B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="30">
-        <f>C26-MIN($B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="D27" s="30">
-        <f>D26-MIN($B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="10" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>BUDGET vs. ACTUAL</t>
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Budget</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Flooring materials</t>
+        </is>
+      </c>
+      <c r="B30" s="12">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,5,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C30" s="12">
+        <f>SUMIF($D$46:$D$145,$A30,$E$46:$E$145)</f>
+        <v/>
+      </c>
+      <c r="D30" s="12">
+        <f>IF(B30="","",B30-C30)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>Flooring materials</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B31" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,5,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,6,FALSE))</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>SUMIF($D$48:$D$147,$A31,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A31,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D31" s="12">
@@ -1548,15 +1541,15 @@
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Underlayment &amp; supplies</t>
+          <t>Stair risers</t>
         </is>
       </c>
       <c r="B32" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,6,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,7,FALSE))</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>SUMIF($D$48:$D$147,$A32,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A32,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D32" s="12">
@@ -1567,15 +1560,15 @@
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Stair nose trim</t>
+          <t>Contractor discount</t>
         </is>
       </c>
       <c r="B33" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,7,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,8,FALSE))</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>SUMIF($D$48:$D$147,$A33,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A33,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D33" s="12">
@@ -1586,15 +1579,15 @@
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Stair risers</t>
+          <t>Sales tax</t>
         </is>
       </c>
       <c r="B34" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,8,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,9,FALSE))</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>SUMIF($D$48:$D$147,$A34,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A34,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D34" s="12">
@@ -1605,15 +1598,15 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Contractor discount</t>
+          <t>Labor — demo &amp; disposal</t>
         </is>
       </c>
       <c r="B35" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,9,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,10,FALSE))</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>SUMIF($D$48:$D$147,$A35,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A35,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D35" s="12">
@@ -1624,15 +1617,15 @@
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Sales tax</t>
+          <t>Labor — install</t>
         </is>
       </c>
       <c r="B36" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,10,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,11,FALSE))</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>SUMIF($D$48:$D$147,$A36,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A36,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D36" s="12">
@@ -1643,15 +1636,15 @@
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Labor — stairs</t>
         </is>
       </c>
       <c r="B37" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,11,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,12,FALSE))</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>SUMIF($D$48:$D$147,$A37,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A37,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D37" s="12">
@@ -1662,15 +1655,12 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Labor — install</t>
-        </is>
-      </c>
-      <c r="B38" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,12,FALSE))</f>
-        <v/>
-      </c>
+          <t>Permits &amp; fees</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n"/>
       <c r="C38" s="12">
-        <f>SUMIF($D$48:$D$147,$A38,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A38,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D38" s="12">
@@ -1681,15 +1671,12 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Labor — stairs</t>
-        </is>
-      </c>
-      <c r="B39" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,13,FALSE))</f>
-        <v/>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="12">
-        <f>SUMIF($D$48:$D$147,$A39,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A39,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D39" s="12">
@@ -1700,113 +1687,99 @@
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Permits &amp; fees</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12">
-        <f>SUMIF($D$48:$D$147,$A40,$E$48:$E$147)</f>
-        <v/>
-      </c>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B40" s="12">
+        <f>SUM(B30:B39)*$B$9</f>
+        <v/>
+      </c>
+      <c r="C40" s="12" t="n"/>
       <c r="D40" s="12">
-        <f>IF(B40="","",B40-C40)</f>
+        <f>B40-C40</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="n"/>
-      <c r="C41" s="12">
-        <f>SUMIF($D$48:$D$147,$A41,$E$48:$E$147)</f>
-        <v/>
-      </c>
-      <c r="D41" s="12">
-        <f>IF(B41="","",B41-C41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B42" s="12">
-        <f>SUM(B31:B41)*$B$9</f>
-        <v/>
-      </c>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12">
-        <f>B42-C42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="A41" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B43" s="31">
-        <f>SUM(B31:B42)</f>
-        <v/>
-      </c>
-      <c r="C43" s="31">
-        <f>SUM(C31:C42)</f>
-        <v/>
-      </c>
-      <c r="D43" s="31">
-        <f>B43-C43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="B41" s="31">
+        <f>SUM(B30:B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="31">
+        <f>SUM(C30:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="31">
+        <f>B41-C41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>COST LOG</t>
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+    </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Vendor</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>Payment method</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A47" s="6" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="n"/>
+      <c r="D47" s="10" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
@@ -2690,45 +2663,26 @@
       <c r="F145" s="10" t="n"/>
       <c r="G145" s="10" t="n"/>
     </row>
-    <row r="146">
-      <c r="A146" s="6" t="n"/>
-      <c r="B146" s="10" t="n"/>
-      <c r="C146" s="10" t="n"/>
-      <c r="D146" s="10" t="n"/>
-      <c r="E146" s="12" t="n"/>
-      <c r="F146" s="10" t="n"/>
-      <c r="G146" s="10" t="n"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="6" t="n"/>
-      <c r="B147" s="10" t="n"/>
-      <c r="C147" s="10" t="n"/>
-      <c r="D147" s="10" t="n"/>
-      <c r="E147" s="12" t="n"/>
-      <c r="F147" s="10" t="n"/>
-      <c r="G147" s="10" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="18">
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="B7:F7"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="B8:F8"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="A46:G46"/>
-    <mergeCell ref="E24:G24"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="E14:G14"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="B10:F10"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
     <mergeCell ref="E20:G20"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2737,8 +2691,8 @@
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=$B$13:$D$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=$A$31:$A$41</formula1>
+    <dataValidation sqref="D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=$A$30:$A$39</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3399,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G147"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3572,7 +3526,7 @@
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>Underlayment &amp; supplies</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B18" s="25" t="inlineStr"/>
@@ -3583,7 +3537,7 @@
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
-          <t>Stair nose trim</t>
+          <t>Stair risers</t>
         </is>
       </c>
       <c r="B19" s="25" t="inlineStr"/>
@@ -3594,30 +3548,39 @@
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
         <is>
-          <t>Stair risers</t>
-        </is>
-      </c>
-      <c r="B20" s="25" t="inlineStr"/>
-      <c r="C20" s="25" t="inlineStr"/>
-      <c r="D20" s="25" t="inlineStr"/>
+          <t>Contractor discount on materials (0%)</t>
+        </is>
+      </c>
+      <c r="B20" s="25">
+        <f>-0.0*SUM(B17:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="25">
+        <f>-0.0*SUM(C17:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="25">
+        <f>-0.0*SUM(D17:D19)</f>
+        <v/>
+      </c>
       <c r="E20" s="10" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
-          <t>Contractor discount on materials (0%)</t>
+          <t>Est. sales tax (6.25% MA, materials)</t>
         </is>
       </c>
       <c r="B21" s="25">
-        <f>-0.0*SUM(B17:B20)</f>
+        <f>SUM(B17:B20)*0.0625</f>
         <v/>
       </c>
       <c r="C21" s="25">
-        <f>-0.0*SUM(C17:C20)</f>
+        <f>SUM(C17:C20)*0.0625</f>
         <v/>
       </c>
       <c r="D21" s="25">
-        <f>-0.0*SUM(D17:D20)</f>
+        <f>SUM(D17:D20)*0.0625</f>
         <v/>
       </c>
       <c r="E21" s="10" t="n"/>
@@ -3625,27 +3588,18 @@
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>Est. sales tax (6.25% MA, materials)</t>
-        </is>
-      </c>
-      <c r="B22" s="25">
-        <f>SUM(B17:B21)*0.0625</f>
-        <v/>
-      </c>
-      <c r="C22" s="25">
-        <f>SUM(C17:C21)*0.0625</f>
-        <v/>
-      </c>
-      <c r="D22" s="25">
-        <f>SUM(D17:D21)*0.0625</f>
-        <v/>
-      </c>
+          <t>Labor — demo &amp; disposal</t>
+        </is>
+      </c>
+      <c r="B22" s="25" t="inlineStr"/>
+      <c r="C22" s="25" t="inlineStr"/>
+      <c r="D22" s="25" t="inlineStr"/>
       <c r="E22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Labor — install</t>
         </is>
       </c>
       <c r="B23" s="25" t="inlineStr"/>
@@ -3656,7 +3610,7 @@
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>Labor — install</t>
+          <t>Labor — stairs (treads &amp; risers)</t>
         </is>
       </c>
       <c r="B24" s="25" t="inlineStr"/>
@@ -3665,97 +3619,105 @@
       <c r="E24" s="10" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="inlineStr">
-        <is>
-          <t>Labor — stairs (treads &amp; risers)</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="inlineStr"/>
-      <c r="C25" s="25" t="inlineStr"/>
-      <c r="D25" s="25" t="inlineStr"/>
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>TOTAL ESTIMATED</t>
+        </is>
+      </c>
+      <c r="B25" s="28">
+        <f>SUM(B17:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="28">
+        <f>SUM(C17:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="28">
+        <f>SUM(D17:D24)</f>
+        <v/>
+      </c>
       <c r="E25" s="10" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
-        <is>
-          <t>TOTAL ESTIMATED</t>
-        </is>
-      </c>
-      <c r="B26" s="28">
-        <f>SUM(B17:B25)</f>
-        <v/>
-      </c>
-      <c r="C26" s="28">
-        <f>SUM(C17:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="28">
-        <f>SUM(D17:D25)</f>
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Premium vs. cheapest option</t>
+        </is>
+      </c>
+      <c r="B26" s="30">
+        <f>B25-MIN($B$25:$D$25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="30">
+        <f>C25-MIN($B$25:$D$25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="30">
+        <f>D25-MIN($B$25:$D$25)</f>
         <v/>
       </c>
       <c r="E26" s="10" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="29" t="inlineStr">
-        <is>
-          <t>Premium vs. cheapest option</t>
-        </is>
-      </c>
-      <c r="B27" s="30">
-        <f>B26-MIN($B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="30">
-        <f>C26-MIN($B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="D27" s="30">
-        <f>D26-MIN($B$26:$D$26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="10" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>BUDGET vs. ACTUAL</t>
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Budget</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>Remaining</t>
-        </is>
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Flooring materials</t>
+        </is>
+      </c>
+      <c r="B30" s="12">
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,5,FALSE))</f>
+        <v/>
+      </c>
+      <c r="C30" s="12">
+        <f>SUMIF($D$46:$D$145,$A30,$E$46:$E$145)</f>
+        <v/>
+      </c>
+      <c r="D30" s="12">
+        <f>IF(B30="","",B30-C30)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>Flooring materials</t>
+          <t>Stair nose trim</t>
         </is>
       </c>
       <c r="B31" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,5,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,6,FALSE))</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>SUMIF($D$48:$D$147,$A31,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A31,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D31" s="12">
@@ -3766,15 +3728,15 @@
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Underlayment &amp; supplies</t>
+          <t>Stair risers</t>
         </is>
       </c>
       <c r="B32" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,6,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,7,FALSE))</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>SUMIF($D$48:$D$147,$A32,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A32,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D32" s="12">
@@ -3785,15 +3747,15 @@
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>Stair nose trim</t>
+          <t>Contractor discount</t>
         </is>
       </c>
       <c r="B33" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,7,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,8,FALSE))</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>SUMIF($D$48:$D$147,$A33,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A33,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D33" s="12">
@@ -3804,15 +3766,15 @@
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Stair risers</t>
+          <t>Sales tax</t>
         </is>
       </c>
       <c r="B34" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,8,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,9,FALSE))</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>SUMIF($D$48:$D$147,$A34,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A34,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D34" s="12">
@@ -3823,15 +3785,15 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Contractor discount</t>
+          <t>Labor — demo &amp; disposal</t>
         </is>
       </c>
       <c r="B35" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,9,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,10,FALSE))</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>SUMIF($D$48:$D$147,$A35,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A35,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D35" s="12">
@@ -3842,15 +3804,15 @@
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Sales tax</t>
+          <t>Labor — install</t>
         </is>
       </c>
       <c r="B36" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,10,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,11,FALSE))</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>SUMIF($D$48:$D$147,$A36,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A36,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D36" s="12">
@@ -3861,15 +3823,15 @@
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Labor — demo &amp; disposal</t>
+          <t>Labor — stairs</t>
         </is>
       </c>
       <c r="B37" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,11,FALSE))</f>
+        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$25,12,FALSE))</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>SUMIF($D$48:$D$147,$A37,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A37,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D37" s="12">
@@ -3880,15 +3842,12 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Labor — install</t>
-        </is>
-      </c>
-      <c r="B38" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,12,FALSE))</f>
-        <v/>
-      </c>
+          <t>Permits &amp; fees</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n"/>
       <c r="C38" s="12">
-        <f>SUMIF($D$48:$D$147,$A38,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A38,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D38" s="12">
@@ -3899,15 +3858,12 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Labor — stairs</t>
-        </is>
-      </c>
-      <c r="B39" s="12">
-        <f>IF($B$8="","",HLOOKUP($B$8,$B$13:$D$26,13,FALSE))</f>
-        <v/>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n"/>
       <c r="C39" s="12">
-        <f>SUMIF($D$48:$D$147,$A39,$E$48:$E$147)</f>
+        <f>SUMIF($D$46:$D$145,$A39,$E$46:$E$145)</f>
         <v/>
       </c>
       <c r="D39" s="12">
@@ -3918,113 +3874,99 @@
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Permits &amp; fees</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="n"/>
-      <c r="C40" s="12">
-        <f>SUMIF($D$48:$D$147,$A40,$E$48:$E$147)</f>
-        <v/>
-      </c>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="B40" s="12">
+        <f>SUM(B30:B39)*$B$9</f>
+        <v/>
+      </c>
+      <c r="C40" s="12" t="n"/>
       <c r="D40" s="12">
-        <f>IF(B40="","",B40-C40)</f>
+        <f>B40-C40</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="n"/>
-      <c r="C41" s="12">
-        <f>SUMIF($D$48:$D$147,$A41,$E$48:$E$147)</f>
-        <v/>
-      </c>
-      <c r="D41" s="12">
-        <f>IF(B41="","",B41-C41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="B42" s="12">
-        <f>SUM(B31:B41)*$B$9</f>
-        <v/>
-      </c>
-      <c r="C42" s="12" t="n"/>
-      <c r="D42" s="12">
-        <f>B42-C42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="A41" s="27" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B43" s="31">
-        <f>SUM(B31:B42)</f>
-        <v/>
-      </c>
-      <c r="C43" s="31">
-        <f>SUM(C31:C42)</f>
-        <v/>
-      </c>
-      <c r="D43" s="31">
-        <f>B43-C43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="B41" s="31">
+        <f>SUM(B30:B40)</f>
+        <v/>
+      </c>
+      <c r="C41" s="31">
+        <f>SUM(C30:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="31">
+        <f>B41-C41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>COST LOG</t>
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Payment method</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+    </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Vendor</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>Payment method</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A47" s="6" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="n"/>
+      <c r="D47" s="10" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
@@ -4908,26 +4850,9 @@
       <c r="F145" s="10" t="n"/>
       <c r="G145" s="10" t="n"/>
     </row>
-    <row r="146">
-      <c r="A146" s="6" t="n"/>
-      <c r="B146" s="10" t="n"/>
-      <c r="C146" s="10" t="n"/>
-      <c r="D146" s="10" t="n"/>
-      <c r="E146" s="12" t="n"/>
-      <c r="F146" s="10" t="n"/>
-      <c r="G146" s="10" t="n"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="6" t="n"/>
-      <c r="B147" s="10" t="n"/>
-      <c r="C147" s="10" t="n"/>
-      <c r="D147" s="10" t="n"/>
-      <c r="E147" s="12" t="n"/>
-      <c r="F147" s="10" t="n"/>
-      <c r="G147" s="10" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A44:G44"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B6:F6"/>
@@ -4936,10 +4861,9 @@
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:G29"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B9:F9"/>
-    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -4948,8 +4872,8 @@
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=$B$13:$D$13</formula1>
     </dataValidation>
-    <dataValidation sqref="D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=$A$31:$A$41</formula1>
+    <dataValidation sqref="D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=$A$30:$A$39</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7004,7 +6928,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>First project. Compare the 3 Floor &amp; Decor plank options (incl. underlayment, stair nose &amp; risers, 5% contractor discount, est. tax, and Footprints labor), pick one in 'Selected option' (yellow cell), and the budget fills in automatically. Log payments in the cost log at the bottom — actuals and the Basis Tracker update themselves.</t>
+          <t>First project. Compare the 3 Floor &amp; Decor plank options (incl. stair nose &amp; risers, 5% contractor discount, est. tax, and Footprints labor), pick one in 'Selected option' (yellow cell), and the budget fills in automatically. Log payments in the cost log at the bottom — actuals and the Basis Tracker update themselves.</t>
         </is>
       </c>
     </row>
@@ -7064,7 +6988,7 @@
       </c>
       <c r="B12" s="34" t="inlineStr">
         <is>
-          <t>For the next project: right-click the tab &gt; Duplicate, rename it, fill in your options/quotes, then add a row in the Basis Tracker improvements table pointing at the new tab's cell C43 (its Actual total).</t>
+          <t>For the next project: right-click the tab &gt; Duplicate, rename it, fill in your options/quotes, then add a row in the Basis Tracker improvements table pointing at the new tab's cell C41 (its Actual total).</t>
         </is>
       </c>
     </row>
@@ -7076,7 +7000,7 @@
       </c>
       <c r="B14" s="34" t="inlineStr">
         <is>
-          <t>Labor: Footprints Floors of Central MA proposal #25584 (6/30/2026) — $9,057.60, materials excluded. Materials: Floor &amp; Decor Waltham cart (7/2026) — Sapelo Shore / Big Sur / Gunstock Oak + Sentinel underlayment (15 rolls), plus 7 stair noses @ $29.99 and 13 risers @ $20; 5% contractor discount on materials.</t>
+          <t>Labor: Footprints Floors of Central MA proposal #25584 (6/30/2026) — $9,057.60, materials excluded. Materials: Floor &amp; Decor Waltham cart (7/2026) — Sapelo Shore / Big Sur / Gunstock Oak (underlayment attached to plank), plus 7 stair noses @ $29.99 and 13 risers @ $20; 5% contractor discount on materials.</t>
         </is>
       </c>
     </row>

</xml_diff>